<commit_message>
lesson16-database p3 mo hinh logic
</commit_message>
<xml_diff>
--- a/Java25 Quyen Phan Database Design.xlsx
+++ b/Java25 Quyen Phan Database Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77148DAC-B5D9-4E45-B083-F5479F5E286F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D978F6-17F5-4875-8A29-83CC5B2DDE4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="283">
   <si>
     <t>MatHang</t>
   </si>
@@ -956,29 +956,184 @@
     <t>MatKhau</t>
   </si>
   <si>
-    <t>1. Xác định tập thực thể</t>
-  </si>
-  <si>
-    <t>2. Xác định thuộc tính của mỗi tập thực thể</t>
-  </si>
-  <si>
-    <t>- Đơn, đa trị, kết hợp, dẫn xuất</t>
-  </si>
-  <si>
-    <t>- Khóa</t>
-  </si>
-  <si>
-    <t>3. Mối kết hợp</t>
-  </si>
-  <si>
-    <t>- Kiểu dữ liệu nguyên tố(không phải là danh sách, đối tượng)</t>
+    <t>Mô hình quan niệm</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đối tượng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của dự án</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>thông tin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cần lưu trữ của từng đối tượng</t>
+    </r>
+  </si>
+  <si>
+    <t>Mô hình logic(trên cơ sở đối tượng, mẫu tin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** KDL nguyên tố(ngày tháng năm, chuỗi, số, luận lý) không thể là danh sách, đối tượng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** Khóa là tập ít nhất các thuộc tính dùng để phân biệt 2/N thực thể khác nhau trong 1 tập thực thể</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** Đảm bảo dữ liệu không trùng nhau, vô nghĩa, tốn vùng nhớ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** Hỗ trợ truy vấn nhanh hơn so với các thuộc tính thông thường</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** Thông qua các cặp số min, max rồi chọn max ở mỗi bên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** Có ba loại mối kết hợp: 11 1n n1 nn, tạo ràng buộc cho các tập thực thể cũng như thiết kế ra CSDL vật lý có thể lưu trữ dữ liệu chính xác</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>thuộc tính</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của mỗi tập thực thể(đơn trị, đa trị, kết hợp, dẫn xuất)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">3. Xác định </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>khóa</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của mỗi tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Xác định</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mối kết hợp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> giữa các tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">    ** https://drive.google.com/file/d/1OpZ1FmAgVQaAvEkpTY1flGrDhtoVJHbA/view?usp=sharing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1078,6 +1233,29 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFFC000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1204,7 +1382,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1343,6 +1521,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1361,23 +1551,10 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1744,13 +1921,13 @@
       <c r="H4" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="I4" s="60" t="s">
+      <c r="I4" s="54" t="s">
         <v>261</v>
       </c>
-      <c r="J4" s="60" t="s">
+      <c r="J4" s="54" t="s">
         <v>262</v>
       </c>
-      <c r="K4" s="60"/>
+      <c r="K4" s="54"/>
     </row>
     <row r="5" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -1871,7 +2048,7 @@
       <c r="C9" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="62" t="s">
+      <c r="D9" s="56" t="s">
         <v>266</v>
       </c>
       <c r="E9" s="2"/>
@@ -1889,7 +2066,7 @@
       <c r="C10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="56" t="s">
         <v>267</v>
       </c>
       <c r="E10" s="2"/>
@@ -1950,7 +2127,7 @@
     </row>
     <row r="14" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
-      <c r="C14" s="63" t="s">
+      <c r="C14" s="57" t="s">
         <v>240</v>
       </c>
       <c r="D14" s="2"/>
@@ -1978,7 +2155,7 @@
     </row>
     <row r="16" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="55" t="s">
         <v>265</v>
       </c>
       <c r="D16" s="2"/>
@@ -2069,7 +2246,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3ED9551-3413-4958-8BF5-9777805D3C81}">
-  <dimension ref="B2:K27"/>
+  <dimension ref="B2:K41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
@@ -2104,13 +2281,13 @@
       <c r="H4" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="I4" s="60" t="s">
+      <c r="I4" s="54" t="s">
         <v>261</v>
       </c>
-      <c r="J4" s="60" t="s">
+      <c r="J4" s="54" t="s">
         <v>262</v>
       </c>
-      <c r="K4" s="60"/>
+      <c r="K4" s="54"/>
     </row>
     <row r="5" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
@@ -2231,7 +2408,7 @@
       <c r="C9" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="62" t="s">
+      <c r="D9" s="56" t="s">
         <v>266</v>
       </c>
       <c r="E9" s="2"/>
@@ -2249,7 +2426,7 @@
       <c r="C10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="56" t="s">
         <v>267</v>
       </c>
       <c r="E10" s="2"/>
@@ -2310,7 +2487,7 @@
     </row>
     <row r="14" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2"/>
-      <c r="C14" s="63" t="s">
+      <c r="C14" s="57" t="s">
         <v>240</v>
       </c>
       <c r="D14" s="2"/>
@@ -2338,7 +2515,7 @@
     </row>
     <row r="16" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
-      <c r="C16" s="61" t="s">
+      <c r="C16" s="55" t="s">
         <v>265</v>
       </c>
       <c r="D16" s="2"/>
@@ -2398,37 +2575,88 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="22" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="64" t="s">
         <v>268</v>
       </c>
-      <c r="C22" s="65"/>
-      <c r="D22" s="65"/>
-      <c r="E22" s="65"/>
-    </row>
-    <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" t="s">
+      <c r="C22" s="64"/>
+    </row>
+    <row r="23" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B23" s="65" t="s">
         <v>269</v>
       </c>
+      <c r="C23" s="65"/>
     </row>
     <row r="24" spans="2:11" s="18" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="66" t="s">
+      <c r="B24" s="65" t="s">
+        <v>270</v>
+      </c>
+      <c r="C24" s="65"/>
+    </row>
+    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B25" s="24"/>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B26" s="24"/>
+    </row>
+    <row r="27" spans="2:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B27" s="64" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B28" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="30" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B31" s="24" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="24" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B26" s="24" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>272</v>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B35" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B36" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B38" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B39" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B40" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B41" t="s">
+        <v>282</v>
       </c>
     </row>
   </sheetData>
@@ -2671,12 +2899,12 @@
       <c r="Q13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="54" t="s">
+      <c r="R13" s="58" t="s">
         <v>68</v>
       </c>
-      <c r="S13" s="54"/>
-      <c r="T13" s="54"/>
-      <c r="U13" s="54"/>
+      <c r="S13" s="58"/>
+      <c r="T13" s="58"/>
+      <c r="U13" s="58"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D14" s="5"/>
@@ -2689,10 +2917,10 @@
       <c r="Q14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="54"/>
-      <c r="S14" s="54"/>
-      <c r="T14" s="54"/>
-      <c r="U14" s="54"/>
+      <c r="R14" s="58"/>
+      <c r="S14" s="58"/>
+      <c r="T14" s="58"/>
+      <c r="U14" s="58"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
@@ -3267,10 +3495,10 @@
       <c r="W18" s="5"/>
     </row>
     <row r="19" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="P19" s="59" t="s">
+      <c r="P19" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="59"/>
+      <c r="Q19" s="63"/>
       <c r="T19" s="4" t="s">
         <v>9</v>
       </c>
@@ -3288,10 +3516,10 @@
       <c r="P20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="58" t="s">
+      <c r="Q20" s="62" t="s">
         <v>14</v>
       </c>
-      <c r="R20" s="58"/>
+      <c r="R20" s="62"/>
       <c r="T20" s="4" t="s">
         <v>94</v>
       </c>
@@ -3309,10 +3537,10 @@
       <c r="P21" s="4">
         <v>1</v>
       </c>
-      <c r="Q21" s="58" t="s">
+      <c r="Q21" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="R21" s="58"/>
+      <c r="R21" s="62"/>
       <c r="T21" s="4" t="s">
         <v>94</v>
       </c>
@@ -3330,10 +3558,10 @@
       <c r="P22" s="4">
         <v>2</v>
       </c>
-      <c r="Q22" s="58" t="s">
+      <c r="Q22" s="62" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="58"/>
+      <c r="R22" s="62"/>
       <c r="T22" s="4" t="s">
         <v>94</v>
       </c>
@@ -3351,10 +3579,10 @@
       <c r="P23" s="4">
         <v>3</v>
       </c>
-      <c r="Q23" s="58" t="s">
+      <c r="Q23" s="62" t="s">
         <v>101</v>
       </c>
-      <c r="R23" s="58"/>
+      <c r="R23" s="62"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
@@ -3373,10 +3601,10 @@
       <c r="P24" s="4">
         <v>4</v>
       </c>
-      <c r="Q24" s="58" t="s">
+      <c r="Q24" s="62" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="58"/>
+      <c r="R24" s="62"/>
       <c r="T24" s="4" t="s">
         <v>95</v>
       </c>
@@ -4021,16 +4249,16 @@
       </c>
     </row>
     <row r="48" spans="3:36" x14ac:dyDescent="0.25">
-      <c r="C48" s="55" t="s">
+      <c r="C48" s="59" t="s">
         <v>220</v>
       </c>
-      <c r="D48" s="56"/>
-      <c r="E48" s="56"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="56"/>
-      <c r="H48" s="56"/>
-      <c r="I48" s="56"/>
-      <c r="J48" s="56"/>
+      <c r="D48" s="60"/>
+      <c r="E48" s="60"/>
+      <c r="F48" s="60"/>
+      <c r="G48" s="60"/>
+      <c r="H48" s="60"/>
+      <c r="I48" s="60"/>
+      <c r="J48" s="60"/>
       <c r="O48" s="29">
         <v>3</v>
       </c>
@@ -4060,16 +4288,16 @@
       </c>
     </row>
     <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="57" t="s">
+      <c r="C49" s="61" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="57"/>
-      <c r="E49" s="57"/>
-      <c r="F49" s="57"/>
-      <c r="G49" s="57"/>
-      <c r="H49" s="57"/>
-      <c r="I49" s="57"/>
-      <c r="J49" s="57"/>
+      <c r="D49" s="61"/>
+      <c r="E49" s="61"/>
+      <c r="F49" s="61"/>
+      <c r="G49" s="61"/>
+      <c r="H49" s="61"/>
+      <c r="I49" s="61"/>
+      <c r="J49" s="61"/>
       <c r="O49" s="29">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
lesson16-database p4 mo hinh logic sua bai
</commit_message>
<xml_diff>
--- a/Java25 Quyen Phan Database Design.xlsx
+++ b/Java25 Quyen Phan Database Design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2349F0B4-8743-4761-8E5D-AFFFCBA778F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF450C49-0F5A-418E-9450-B44F448DD5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,6 +34,30 @@
     <author>Quyen Ngoc Phan</author>
   </authors>
   <commentList>
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{C541F4FB-5C59-473A-9FDC-3FEA134C8F1E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+NhanVien của cửa hàng</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="I7" authorId="0" shapeId="0" xr:uid="{3D2FB91A-2B49-46BC-B762-B0D688FB2C36}">
       <text>
         <r>
@@ -130,7 +154,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{112469D1-2108-4234-A21A-01AC70F1FE5A}">
+    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{4CCC5A17-BB52-4B86-AAF8-F83EBFA67059}">
       <text>
         <r>
           <rPr>
@@ -202,36 +226,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{4CCC5A17-BB52-4B86-AAF8-F83EBFA67059}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Quyen Ngoc Phan:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Thuộc tính dẫn xuất</t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="315">
   <si>
     <t>MatHang</t>
   </si>
@@ -1381,12 +1381,57 @@
   <si>
     <t>MaPTTT</t>
   </si>
+  <si>
+    <t>TTDX trong MatHang</t>
+  </si>
+  <si>
+    <t>MaCL</t>
+  </si>
+  <si>
+    <t>MaHA</t>
+  </si>
+  <si>
+    <t>DuongdanHA</t>
+  </si>
+  <si>
+    <t>SoDienThoai</t>
+  </si>
+  <si>
+    <t>MXH_TaiKhoan</t>
+  </si>
+  <si>
+    <t>MXH_MaDangNhap</t>
+  </si>
+  <si>
+    <t>TrangThaiDonHang</t>
+  </si>
+  <si>
+    <t>Chờ xử lý</t>
+  </si>
+  <si>
+    <t>Đã tiếp nhận</t>
+  </si>
+  <si>
+    <t>Giao hàng thành công</t>
+  </si>
+  <si>
+    <t>Enum</t>
+  </si>
+  <si>
+    <t>MaTTDH</t>
+  </si>
+  <si>
+    <t>Kết hợp</t>
+  </si>
+  <si>
+    <t>ChiTietTrangThaiDonHang</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1540,6 +1585,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -1662,7 +1714,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1819,6 +1871,18 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1837,19 +1901,10 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2541,20 +2596,36 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3ED9551-3413-4958-8BF5-9777805D3C81}">
-  <dimension ref="B2:L41"/>
+  <dimension ref="A2:O41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="16" width="20.7109375" customWidth="1"/>
-    <col min="17" max="20" width="12.7109375" customWidth="1"/>
+    <col min="2" max="5" width="20.7109375" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" customWidth="1"/>
+    <col min="7" max="17" width="20.7109375" customWidth="1"/>
+    <col min="18" max="21" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F3" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="J3" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="K3" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="L3" s="49" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>0</v>
       </c>
@@ -2568,7 +2639,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>250</v>
+        <v>314</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>254</v>
@@ -2585,45 +2656,69 @@
       <c r="K4" s="1" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="5" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="67" t="s">
+      <c r="L4" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="60" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="66" t="s">
+      <c r="E5" s="60" t="s">
         <v>283</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="2" t="s">
+      <c r="F5" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="60" t="s">
         <v>255</v>
       </c>
-      <c r="H5" s="67" t="s">
+      <c r="H5" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="I5" s="67" t="s">
+      <c r="I5" s="60" t="s">
         <v>288</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="60" t="s">
         <v>290</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="60" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="6" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L5" s="60" t="s">
+        <v>312</v>
+      </c>
+      <c r="M5" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O5" s="60" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>7</v>
+      <c r="C6" s="57" t="s">
+        <v>6</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>241</v>
@@ -2631,8 +2726,8 @@
       <c r="E6" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>251</v>
+      <c r="F6" s="15" t="s">
+        <v>307</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>256</v>
@@ -2649,13 +2744,25 @@
       <c r="K6" s="2" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="7" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="57" t="s">
         <v>292</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>242</v>
@@ -2663,7 +2770,7 @@
       <c r="E7" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="57" t="s">
         <v>252</v>
       </c>
       <c r="G7" s="2"/>
@@ -2675,19 +2782,28 @@
         <v>14</v>
       </c>
       <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="70" t="s">
+        <v>300</v>
+      </c>
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>243</v>
+        <v>304</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>248</v>
+        <v>304</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>18</v>
@@ -2697,36 +2813,42 @@
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>236</v>
+        <v>10</v>
       </c>
       <c r="D9" s="56" t="s">
-        <v>266</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>249</v>
-      </c>
+        <v>305</v>
+      </c>
+      <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
       <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
         <v>230</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>10</v>
+        <v>297</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>267</v>
+        <v>306</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -2735,15 +2857,21 @@
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="69" t="s">
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="62" t="s">
         <v>295</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="C11" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>190</v>
+      </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -2751,13 +2879,17 @@
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="69" t="s">
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="62" t="s">
         <v>296</v>
       </c>
-      <c r="C12" s="70" t="s">
-        <v>238</v>
+      <c r="C12" s="2" t="s">
+        <v>239</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2767,13 +2899,17 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="69" t="s">
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="62" t="s">
         <v>294</v>
       </c>
-      <c r="C13" s="57" t="s">
-        <v>298</v>
+      <c r="C13" s="63" t="s">
+        <v>240</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2783,13 +2919,17 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="57" t="s">
         <v>284</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>239</v>
+      <c r="C14" s="57" t="s">
+        <v>253</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -2799,14 +2939,16 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
       <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="57" t="s">
         <v>285</v>
       </c>
-      <c r="C15" s="70" t="s">
-        <v>240</v>
-      </c>
+      <c r="C15" s="57"/>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -2815,12 +2957,14 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
-    </row>
-    <row r="16" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2"/>
-      <c r="C16" s="57" t="s">
-        <v>253</v>
-      </c>
+      <c r="C16" s="2"/>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -2829,12 +2973,14 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2"/>
-      <c r="C17" s="57" t="s">
-        <v>6</v>
-      </c>
+      <c r="C17" s="57"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
@@ -2843,8 +2989,12 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
-    </row>
-    <row r="18" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -2855,8 +3005,12 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
-    </row>
-    <row r="19" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -2867,8 +3021,12 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
-    </row>
-    <row r="20" spans="2:12" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -2879,8 +3037,12 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
-    </row>
-    <row r="22" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="22" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="58" t="s">
         <v>268</v>
       </c>
@@ -2894,8 +3056,11 @@
       <c r="I22" s="52" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="23" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J22" s="71" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="23" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B23" s="59" t="s">
         <v>269</v>
       </c>
@@ -2909,10 +3074,13 @@
       <c r="I23" t="s">
         <v>288</v>
       </c>
-      <c r="J23" s="49"/>
+      <c r="J23" s="49" t="s">
+        <v>309</v>
+      </c>
       <c r="K23" s="49"/>
-    </row>
-    <row r="24" spans="2:12" s="18" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L23" s="49"/>
+    </row>
+    <row r="24" spans="2:15" s="18" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="59" t="s">
         <v>270</v>
       </c>
@@ -2926,22 +3094,31 @@
       <c r="I24" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="J24" s="49"/>
+      <c r="J24" s="49" t="s">
+        <v>100</v>
+      </c>
       <c r="K24" s="49"/>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="L24" s="49"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B25" s="24"/>
       <c r="G25" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="J25" s="49" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B26" s="24"/>
       <c r="G26" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="27" spans="2:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="J26" s="49" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="27" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B27" s="58" t="s">
         <v>271</v>
       </c>
@@ -2949,16 +3126,16 @@
         <v>286</v>
       </c>
     </row>
-    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>279</v>
       </c>
-      <c r="G30" s="67" t="s">
+      <c r="G30" s="60" t="s">
         <v>1</v>
       </c>
       <c r="H30" s="2" t="s">
@@ -2973,11 +3150,12 @@
       <c r="K30" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L30" s="2" t="s">
+      <c r="L30" s="2"/>
+      <c r="M30" s="2" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B31" s="24" t="s">
         <v>272</v>
       </c>
@@ -2990,29 +3168,33 @@
       <c r="I31" s="49" t="s">
         <v>293</v>
       </c>
-      <c r="J31" s="49"/>
+      <c r="J31" s="49">
+        <v>112</v>
+      </c>
       <c r="K31" s="49">
         <v>120</v>
       </c>
-      <c r="L31" s="49">
+      <c r="L31" s="49"/>
+      <c r="M31" s="49">
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="G32" s="68">
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="G32" s="61">
         <v>2</v>
       </c>
-      <c r="H32" s="68" t="s">
+      <c r="H32" s="61" t="s">
         <v>287</v>
       </c>
-      <c r="I32" s="68" t="s">
+      <c r="I32" s="61" t="s">
         <v>85</v>
       </c>
-      <c r="J32" s="68"/>
-      <c r="K32" s="68">
+      <c r="J32" s="61"/>
+      <c r="K32" s="61">
         <v>122</v>
       </c>
-      <c r="L32" s="68">
+      <c r="L32" s="61"/>
+      <c r="M32" s="61">
         <v>5</v>
       </c>
     </row>
@@ -3297,12 +3479,12 @@
       <c r="Q13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="60" t="s">
+      <c r="R13" s="64" t="s">
         <v>68</v>
       </c>
-      <c r="S13" s="60"/>
-      <c r="T13" s="60"/>
-      <c r="U13" s="60"/>
+      <c r="S13" s="64"/>
+      <c r="T13" s="64"/>
+      <c r="U13" s="64"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D14" s="5"/>
@@ -3315,10 +3497,10 @@
       <c r="Q14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="60"/>
-      <c r="S14" s="60"/>
-      <c r="T14" s="60"/>
-      <c r="U14" s="60"/>
+      <c r="R14" s="64"/>
+      <c r="S14" s="64"/>
+      <c r="T14" s="64"/>
+      <c r="U14" s="64"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
@@ -3893,10 +4075,10 @@
       <c r="W18" s="5"/>
     </row>
     <row r="19" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="P19" s="65" t="s">
+      <c r="P19" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="65"/>
+      <c r="Q19" s="69"/>
       <c r="T19" s="4" t="s">
         <v>9</v>
       </c>
@@ -3914,10 +4096,10 @@
       <c r="P20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="64" t="s">
+      <c r="Q20" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="R20" s="64"/>
+      <c r="R20" s="68"/>
       <c r="T20" s="4" t="s">
         <v>94</v>
       </c>
@@ -3935,10 +4117,10 @@
       <c r="P21" s="4">
         <v>1</v>
       </c>
-      <c r="Q21" s="64" t="s">
+      <c r="Q21" s="68" t="s">
         <v>99</v>
       </c>
-      <c r="R21" s="64"/>
+      <c r="R21" s="68"/>
       <c r="T21" s="4" t="s">
         <v>94</v>
       </c>
@@ -3956,10 +4138,10 @@
       <c r="P22" s="4">
         <v>2</v>
       </c>
-      <c r="Q22" s="64" t="s">
+      <c r="Q22" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="64"/>
+      <c r="R22" s="68"/>
       <c r="T22" s="4" t="s">
         <v>94</v>
       </c>
@@ -3977,10 +4159,10 @@
       <c r="P23" s="4">
         <v>3</v>
       </c>
-      <c r="Q23" s="64" t="s">
+      <c r="Q23" s="68" t="s">
         <v>101</v>
       </c>
-      <c r="R23" s="64"/>
+      <c r="R23" s="68"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
@@ -3999,10 +4181,10 @@
       <c r="P24" s="4">
         <v>4</v>
       </c>
-      <c r="Q24" s="64" t="s">
+      <c r="Q24" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="64"/>
+      <c r="R24" s="68"/>
       <c r="T24" s="4" t="s">
         <v>95</v>
       </c>
@@ -4647,16 +4829,16 @@
       </c>
     </row>
     <row r="48" spans="3:36" x14ac:dyDescent="0.25">
-      <c r="C48" s="61" t="s">
+      <c r="C48" s="65" t="s">
         <v>220</v>
       </c>
-      <c r="D48" s="62"/>
-      <c r="E48" s="62"/>
-      <c r="F48" s="62"/>
-      <c r="G48" s="62"/>
-      <c r="H48" s="62"/>
-      <c r="I48" s="62"/>
-      <c r="J48" s="62"/>
+      <c r="D48" s="66"/>
+      <c r="E48" s="66"/>
+      <c r="F48" s="66"/>
+      <c r="G48" s="66"/>
+      <c r="H48" s="66"/>
+      <c r="I48" s="66"/>
+      <c r="J48" s="66"/>
       <c r="O48" s="29">
         <v>3</v>
       </c>
@@ -4686,16 +4868,16 @@
       </c>
     </row>
     <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="63" t="s">
+      <c r="C49" s="67" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="63"/>
-      <c r="E49" s="63"/>
-      <c r="F49" s="63"/>
-      <c r="G49" s="63"/>
-      <c r="H49" s="63"/>
-      <c r="I49" s="63"/>
-      <c r="J49" s="63"/>
+      <c r="D49" s="67"/>
+      <c r="E49" s="67"/>
+      <c r="F49" s="67"/>
+      <c r="G49" s="67"/>
+      <c r="H49" s="67"/>
+      <c r="I49" s="67"/>
+      <c r="J49" s="67"/>
       <c r="O49" s="29">
         <v>4</v>
       </c>

</xml_diff>

<commit_message>
lesson16-database p5 mo hinh quan he
</commit_message>
<xml_diff>
--- a/Java25 Quyen Phan Database Design.xlsx
+++ b/Java25 Quyen Phan Database Design.xlsx
@@ -1,28 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF450C49-0F5A-418E-9450-B44F448DD5B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66D44D56-031A-49DF-A0E2-7F0D6111CE64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
     <sheet name="2. Mô hình logic" sheetId="5" r:id="rId2"/>
-    <sheet name="ERD - Mô hình logic" sheetId="2" r:id="rId3"/>
-    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId4"/>
-    <sheet name="DB - Mô hình vật lý" sheetId="4" r:id="rId5"/>
+    <sheet name="3. Mô hình quan hệ" sheetId="6" r:id="rId3"/>
+    <sheet name="ERD - Mô hình logic" sheetId="2" r:id="rId4"/>
+    <sheet name="RD - Mô hình quan hệ" sheetId="3" r:id="rId5"/>
+    <sheet name="DB - Mô hình vật lý" sheetId="4" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -230,8 +242,282 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Quyen Ngoc Phan</author>
+  </authors>
+  <commentList>
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{22E46641-A935-4FE4-A7CD-80C5D7DB30FD}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+NhanVien của cửa hàng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{2DA2E551-DE99-48A5-9D67-5E8DC61248E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+LoaiHangPhu thuộc LoaiHang</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="0" shapeId="0" xr:uid="{A832552A-A362-4139-BA16-11FC431FA314}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Muốn lưu trữ lịch sử giá mua từ các nhà cung cấp theo thời gian</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{26FC4D9F-5193-4274-AA9B-7B20D50002C9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+GiaBan phụ thuộc vào KichThuoc</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{B991BA08-95ED-4BA0-8652-FD2EC8009C23}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Lưu trữ theo MatHang, KichThuoc</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{871AE503-040D-4F5E-AFE8-67ED97E07A32}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Thuộc tính dẫn xuất</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0" xr:uid="{C5E22E80-59E4-4118-830C-EE48E603F271}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+MatHang thuộc trực tiếp LoaiHang || thông qua LoaiHangPhu mới đến LoaiHang, nullable</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0" xr:uid="{C62CADBE-F98D-418B-BEA1-A7213E8CDF49}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+xem chỗ LoaiHang</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{8CB493CD-E43C-4813-8551-B25538B62201}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+0/1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J63" authorId="0" shapeId="0" xr:uid="{66270A31-718B-4FD0-9656-385D47CCEF1C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+0/1</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J81" authorId="0" shapeId="0" xr:uid="{D8DB9340-3666-4F98-A39A-F300535D9AB5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+0/1</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="630" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="414">
   <si>
     <t>MatHang</t>
   </si>
@@ -1426,12 +1712,449 @@
   <si>
     <t>ChiTietTrangThaiDonHang</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>đối tượng</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của dự án</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>thông tin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> cần lưu trữ của từng đối tượng</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. Xác định các </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>thuộc tính</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của mỗi tập thực thể(đơn trị, đa trị, kết hợp, dẫn xuất)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">3. Xác định </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>khóa</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> của mỗi tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Xác định</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mối kết hợp</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> giữa các tập thực thể</t>
+    </r>
+  </si>
+  <si>
+    <t>Mô hình quan hệ(hình thành cơ sở dữ liệu vật lý)</t>
+  </si>
+  <si>
+    <t>1. Tập thực thể</t>
+  </si>
+  <si>
+    <t>==</t>
+  </si>
+  <si>
+    <t>2. Thuộc tính</t>
+  </si>
+  <si>
+    <t>3. Khóa(s) (được chọn)</t>
+  </si>
+  <si>
+    <t>4. Mối kết hợp</t>
+  </si>
+  <si>
+    <t>4. Giải thích công thức từ "Mối kết hợp" 11 1nn1 nn từ mô hình logic để tạo ra các "khóa ngoại" trong mô hình quan hệ</t>
+  </si>
+  <si>
+    <t>TH1</t>
+  </si>
+  <si>
+    <t>Quan hệ 1-N N-1</t>
+  </si>
+  <si>
+    <t>MH A1</t>
+  </si>
+  <si>
+    <t>Áo</t>
+  </si>
+  <si>
+    <t>Xanh</t>
+  </si>
+  <si>
+    <t>MH A2</t>
+  </si>
+  <si>
+    <t>Quần</t>
+  </si>
+  <si>
+    <t>Đỏ</t>
+  </si>
+  <si>
+    <t>MH A3</t>
+  </si>
+  <si>
+    <t>Giày dép</t>
+  </si>
+  <si>
+    <t>Đen</t>
+  </si>
+  <si>
+    <t>LH1</t>
+  </si>
+  <si>
+    <t>Loại Hàng 1</t>
+  </si>
+  <si>
+    <t>LH2</t>
+  </si>
+  <si>
+    <t>Loại Hàng 2</t>
+  </si>
+  <si>
+    <t>LH3</t>
+  </si>
+  <si>
+    <t>Loại Hàng 3</t>
+  </si>
+  <si>
+    <t>LH4</t>
+  </si>
+  <si>
+    <t>Loại Hàng 4</t>
+  </si>
+  <si>
+    <t>Bài toán: [1] LoaiHang [N] MatHang</t>
+  </si>
+  <si>
+    <t>Câu hỏi: Tạo khóa ngoại, tạo ở đâu ?</t>
+  </si>
+  <si>
+    <t>MH A4</t>
+  </si>
+  <si>
+    <t>Mũ</t>
+  </si>
+  <si>
+    <t>Tím</t>
+  </si>
+  <si>
+    <t>Khóa chính</t>
+  </si>
+  <si>
+    <t>- 1 table chỉ có duy nhất 1 khóa chính</t>
+  </si>
+  <si>
+    <t>- 1 khóa chính có thể có 1/N columns</t>
+  </si>
+  <si>
+    <t>- Dữ liệu not nullable, không được trùng nhau</t>
+  </si>
+  <si>
+    <t>- Dữ liệu nullable nhưng mà thường là not nullable để trỏ đến not nullable từ khóa chính ở bảng tham chiếu</t>
+  </si>
+  <si>
+    <t>- Được phép trùng nhau</t>
+  </si>
+  <si>
+    <t>- Miền giá trị phải trùng với khóa chính</t>
+  </si>
+  <si>
+    <t>Bảng 1 = Bảng cha</t>
+  </si>
+  <si>
+    <t>Bảng N = Bảng con</t>
+  </si>
+  <si>
+    <t>Referenced Table</t>
+  </si>
+  <si>
+    <t>Referencing Table</t>
+  </si>
+  <si>
+    <t>Bị tham chiếu</t>
+  </si>
+  <si>
+    <t>Tham chiếu</t>
+  </si>
+  <si>
+    <t>Lưu ý:</t>
+  </si>
+  <si>
+    <t>- Nếu bảng cha có khóa chính là 1 column, bảng con tạo ra 1 column làm khóa ngoại</t>
+  </si>
+  <si>
+    <t>DH 1</t>
+  </si>
+  <si>
+    <t>DH 2</t>
+  </si>
+  <si>
+    <t>SoLuongMua</t>
+  </si>
+  <si>
+    <t>DH 5</t>
+  </si>
+  <si>
+    <t>Bảng 1</t>
+  </si>
+  <si>
+    <t>Bảng N</t>
+  </si>
+  <si>
+    <t>MaCTMH</t>
+  </si>
+  <si>
+    <t>Unique Constraint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lý thuyết: </t>
+  </si>
+  <si>
+    <t>- Cách 1: Quan hệ 1 N thì bỏ 1 vào N nghĩa là column khóa ngoại sẽ được tạo bên bảng N rồi tạo liên kết đến khóa chính bên bảng 1</t>
+  </si>
+  <si>
+    <t>LoaiMatHang</t>
+  </si>
+  <si>
+    <t>MaLH [FK]</t>
+  </si>
+  <si>
+    <t>MH A5</t>
+  </si>
+  <si>
+    <t>Thắt lưng</t>
+  </si>
+  <si>
+    <t>Da</t>
+  </si>
+  <si>
+    <t>Unique: Đảm bảo dữ liệu không trùng</t>
+  </si>
+  <si>
+    <t>- Đảm bảo dữ liệu không trùng, not nullable</t>
+  </si>
+  <si>
+    <t>- Hỗ trợ truy vấn nhanh hơn khi tìm kiếm</t>
+  </si>
+  <si>
+    <t>- Bị tham chiếu bởi các FK từ table khác</t>
+  </si>
+  <si>
+    <t>Primary key</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">MaMH [FK] Unique | </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF0070C0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>PK</t>
+    </r>
+  </si>
+  <si>
+    <t>- Cách 2: Quan hệ 1 N, tạo ra một table kết hợp có columns là khóa ngoại trỏ đến 2/N tables cha, FK mà liên kết đến bảng N thì cho là là PK</t>
+  </si>
+  <si>
+    <t>Cách làm số 2 trong quan hệ 1 N</t>
+  </si>
+  <si>
+    <t>(*)</t>
+  </si>
+  <si>
+    <t>(**)</t>
+  </si>
+  <si>
+    <t>(***)</t>
+  </si>
+  <si>
+    <t>(****)</t>
+  </si>
+  <si>
+    <t>- Nếu bảng cha có khóa chính là N column, bảng con tạo ra N column làm khóa ngoại =&gt; xử lý</t>
+  </si>
+  <si>
+    <t>TH: Khóa ngoại liên kết đến khóa chính trong cùng một table</t>
+  </si>
+  <si>
+    <t>NV 1</t>
+  </si>
+  <si>
+    <t>NV 2</t>
+  </si>
+  <si>
+    <t>NV 3</t>
+  </si>
+  <si>
+    <t>NV 4</t>
+  </si>
+  <si>
+    <t>NV 5</t>
+  </si>
+  <si>
+    <t>NV 6</t>
+  </si>
+  <si>
+    <t>NV 7</t>
+  </si>
+  <si>
+    <t>NV 8</t>
+  </si>
+  <si>
+    <t>MaNQL</t>
+  </si>
+  <si>
+    <t>Họ Tên 1</t>
+  </si>
+  <si>
+    <t>Họ Tên 2</t>
+  </si>
+  <si>
+    <t>Họ Tên 3</t>
+  </si>
+  <si>
+    <t>Họ Tên 4</t>
+  </si>
+  <si>
+    <t>Họ Tên 5</t>
+  </si>
+  <si>
+    <t>Họ Tên 6</t>
+  </si>
+  <si>
+    <t>Họ Tên 7</t>
+  </si>
+  <si>
+    <t>Họ Tên 8</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="31" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1592,8 +2315,73 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1666,8 +2454,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1710,11 +2504,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1883,6 +2697,9 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1901,11 +2718,68 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2790,7 +3664,7 @@
       <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="70" t="s">
+      <c r="A8" s="64" t="s">
         <v>300</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -3056,7 +3930,7 @@
       <c r="I22" s="52" t="s">
         <v>285</v>
       </c>
-      <c r="J22" s="71" t="s">
+      <c r="J22" s="49" t="s">
         <v>308</v>
       </c>
     </row>
@@ -3246,6 +4120,1948 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA1D6412-D11D-457E-8A24-4F747CD8558C}">
+  <dimension ref="A2:O115"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" style="75" customWidth="1"/>
+    <col min="2" max="5" width="20.7109375" style="75" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="75" customWidth="1"/>
+    <col min="7" max="17" width="20.7109375" style="75" customWidth="1"/>
+    <col min="18" max="21" width="12.7109375" style="75" customWidth="1"/>
+    <col min="22" max="16384" width="9.140625" style="75"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D2" s="75" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="F3" s="49" t="s">
+        <v>313</v>
+      </c>
+      <c r="J3" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="K3" s="49" t="s">
+        <v>311</v>
+      </c>
+      <c r="L3" s="49" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="60" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="60" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="60" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="60" t="s">
+        <v>283</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="60" t="s">
+        <v>255</v>
+      </c>
+      <c r="H5" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="60" t="s">
+        <v>288</v>
+      </c>
+      <c r="J5" s="60" t="s">
+        <v>290</v>
+      </c>
+      <c r="K5" s="60" t="s">
+        <v>299</v>
+      </c>
+      <c r="L5" s="60" t="s">
+        <v>312</v>
+      </c>
+      <c r="M5" s="60" t="s">
+        <v>301</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O5" s="60" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="57" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>307</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="57" t="s">
+        <v>292</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="F7" s="57" t="s">
+        <v>252</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="57" t="s">
+        <v>284</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="O7" s="2"/>
+    </row>
+    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="64" t="s">
+        <v>300</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+    </row>
+    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="56" t="s">
+        <v>305</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+    </row>
+    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D10" s="56" t="s">
+        <v>306</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+    </row>
+    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="62" t="s">
+        <v>295</v>
+      </c>
+      <c r="C11" s="57" t="s">
+        <v>298</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+    </row>
+    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="62" t="s">
+        <v>296</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+    </row>
+    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="62" t="s">
+        <v>294</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="57" t="s">
+        <v>284</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>253</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+    </row>
+    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="57" t="s">
+        <v>285</v>
+      </c>
+      <c r="C15" s="57"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+    </row>
+    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+    </row>
+    <row r="17" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+    </row>
+    <row r="18" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+    </row>
+    <row r="19" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+    </row>
+    <row r="20" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+    </row>
+    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B22" s="71" t="s">
+        <v>268</v>
+      </c>
+      <c r="C22" s="71"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="77"/>
+      <c r="H22" s="77"/>
+      <c r="I22" s="77"/>
+      <c r="J22" s="49"/>
+    </row>
+    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B23" s="72" t="s">
+        <v>315</v>
+      </c>
+      <c r="C23" s="72"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="76"/>
+      <c r="I23" s="76"/>
+      <c r="J23" s="49"/>
+      <c r="K23" s="49"/>
+      <c r="L23" s="49"/>
+    </row>
+    <row r="24" spans="2:15" s="18" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="72" t="s">
+        <v>316</v>
+      </c>
+      <c r="C24" s="72"/>
+      <c r="D24" s="72"/>
+      <c r="E24" s="72"/>
+      <c r="F24" s="72"/>
+      <c r="G24" s="72"/>
+      <c r="H24" s="72"/>
+      <c r="I24" s="72"/>
+      <c r="J24" s="49"/>
+      <c r="K24" s="49"/>
+      <c r="L24" s="49"/>
+    </row>
+    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B25" s="78"/>
+      <c r="C25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="76"/>
+      <c r="I25" s="76"/>
+      <c r="J25" s="49"/>
+    </row>
+    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B26" s="78"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="76"/>
+      <c r="E26" s="76"/>
+      <c r="F26" s="76"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="76"/>
+      <c r="I26" s="76"/>
+      <c r="J26" s="49"/>
+    </row>
+    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B27" s="71" t="s">
+        <v>271</v>
+      </c>
+      <c r="C27" s="76"/>
+      <c r="D27" s="76"/>
+      <c r="E27" s="76"/>
+      <c r="F27" s="76"/>
+      <c r="G27" s="76"/>
+      <c r="H27" s="76"/>
+      <c r="I27" s="76"/>
+    </row>
+    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B28" s="76" t="s">
+        <v>317</v>
+      </c>
+      <c r="C28" s="76"/>
+      <c r="D28" s="76"/>
+      <c r="E28" s="76"/>
+      <c r="F28" s="76"/>
+      <c r="G28" s="76"/>
+      <c r="H28" s="76"/>
+      <c r="I28" s="76"/>
+    </row>
+    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B29" s="76"/>
+      <c r="C29" s="76"/>
+      <c r="D29" s="76"/>
+      <c r="E29" s="76"/>
+      <c r="F29" s="76"/>
+      <c r="G29" s="76"/>
+      <c r="H29" s="76"/>
+      <c r="I29" s="76"/>
+    </row>
+    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B30" s="76" t="s">
+        <v>318</v>
+      </c>
+      <c r="C30" s="76"/>
+      <c r="D30" s="76"/>
+      <c r="E30" s="76"/>
+      <c r="F30" s="76"/>
+      <c r="G30" s="76"/>
+      <c r="H30" s="76"/>
+      <c r="I30" s="76"/>
+    </row>
+    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B31" s="78" t="s">
+        <v>272</v>
+      </c>
+      <c r="C31" s="76"/>
+      <c r="D31" s="76"/>
+      <c r="E31" s="76"/>
+      <c r="F31" s="76"/>
+      <c r="G31" s="76"/>
+      <c r="H31" s="76"/>
+      <c r="I31" s="76"/>
+    </row>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
+      <c r="B32" s="76"/>
+      <c r="C32" s="76"/>
+      <c r="D32" s="76"/>
+      <c r="E32" s="76"/>
+      <c r="F32" s="76"/>
+      <c r="G32" s="73"/>
+      <c r="H32" s="73"/>
+      <c r="I32" s="73"/>
+      <c r="J32" s="61"/>
+      <c r="K32" s="61"/>
+      <c r="L32" s="61"/>
+      <c r="M32" s="61"/>
+    </row>
+    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B33" s="76" t="s">
+        <v>319</v>
+      </c>
+      <c r="C33" s="76"/>
+      <c r="D33" s="76"/>
+      <c r="E33" s="76"/>
+      <c r="F33" s="76"/>
+      <c r="G33" s="76"/>
+      <c r="H33" s="76" t="s">
+        <v>352</v>
+      </c>
+      <c r="I33" s="76"/>
+    </row>
+    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B34" s="76" t="s">
+        <v>273</v>
+      </c>
+      <c r="C34" s="76"/>
+      <c r="D34" s="76"/>
+      <c r="E34" s="76"/>
+      <c r="F34" s="76"/>
+      <c r="G34" s="76"/>
+      <c r="H34" s="78" t="s">
+        <v>355</v>
+      </c>
+      <c r="I34" s="76"/>
+    </row>
+    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B35" s="76" t="s">
+        <v>274</v>
+      </c>
+      <c r="C35" s="76"/>
+      <c r="D35" s="76"/>
+      <c r="E35" s="76"/>
+      <c r="F35" s="76"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="78" t="s">
+        <v>353</v>
+      </c>
+      <c r="I35" s="76"/>
+    </row>
+    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B36" s="76" t="s">
+        <v>275</v>
+      </c>
+      <c r="C36" s="76"/>
+      <c r="D36" s="76"/>
+      <c r="E36" s="76"/>
+      <c r="F36" s="76"/>
+      <c r="G36" s="76"/>
+      <c r="H36" s="78" t="s">
+        <v>354</v>
+      </c>
+      <c r="I36" s="76"/>
+    </row>
+    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B37" s="76"/>
+      <c r="C37" s="76"/>
+      <c r="D37" s="76"/>
+      <c r="E37" s="76"/>
+      <c r="F37" s="76"/>
+      <c r="G37" s="76"/>
+      <c r="H37" s="76"/>
+      <c r="I37" s="76"/>
+    </row>
+    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B38" s="76" t="s">
+        <v>320</v>
+      </c>
+      <c r="C38" s="76"/>
+      <c r="D38" s="76"/>
+      <c r="E38" s="76"/>
+      <c r="F38" s="76"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="76" t="s">
+        <v>136</v>
+      </c>
+      <c r="I38" s="76"/>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B39" s="76" t="s">
+        <v>276</v>
+      </c>
+      <c r="C39" s="76"/>
+      <c r="D39" s="76"/>
+      <c r="E39" s="76"/>
+      <c r="F39" s="76"/>
+      <c r="G39" s="76"/>
+      <c r="H39" s="78" t="s">
+        <v>356</v>
+      </c>
+      <c r="I39" s="76"/>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="76" t="s">
+        <v>277</v>
+      </c>
+      <c r="C40" s="76"/>
+      <c r="D40" s="76"/>
+      <c r="E40" s="76"/>
+      <c r="F40" s="76"/>
+      <c r="G40" s="76"/>
+      <c r="H40" s="78" t="s">
+        <v>357</v>
+      </c>
+      <c r="I40" s="76"/>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="76" t="s">
+        <v>282</v>
+      </c>
+      <c r="C41" s="76"/>
+      <c r="D41" s="76"/>
+      <c r="E41" s="76"/>
+      <c r="F41" s="76"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="78" t="s">
+        <v>358</v>
+      </c>
+      <c r="I41" s="76"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="76"/>
+      <c r="C42" s="76"/>
+      <c r="D42" s="76"/>
+      <c r="E42" s="76"/>
+      <c r="F42" s="76"/>
+      <c r="G42" s="76"/>
+      <c r="H42" s="76"/>
+      <c r="I42" s="76"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="76"/>
+      <c r="C43" s="76"/>
+      <c r="D43" s="76"/>
+      <c r="E43" s="76"/>
+      <c r="F43" s="76"/>
+      <c r="G43" s="76"/>
+      <c r="H43" s="76"/>
+      <c r="I43" s="76"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="C44" s="76"/>
+      <c r="D44" s="76"/>
+      <c r="E44" s="76"/>
+      <c r="F44" s="76"/>
+      <c r="G44" s="76"/>
+      <c r="H44" s="76"/>
+      <c r="I44" s="76"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="76" t="s">
+        <v>322</v>
+      </c>
+      <c r="C45" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="D45" s="76" t="s">
+        <v>78</v>
+      </c>
+      <c r="E45" s="76"/>
+      <c r="F45" s="76"/>
+      <c r="G45" s="76"/>
+      <c r="H45" s="76"/>
+      <c r="I45" s="76"/>
+    </row>
+    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B46" s="76" t="s">
+        <v>324</v>
+      </c>
+      <c r="C46" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="D46" s="76" t="s">
+        <v>79</v>
+      </c>
+      <c r="E46" s="76"/>
+      <c r="F46" s="76"/>
+      <c r="G46" s="76"/>
+      <c r="H46" s="76"/>
+      <c r="I46" s="76"/>
+    </row>
+    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B47" s="76" t="s">
+        <v>325</v>
+      </c>
+      <c r="C47" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="D47" s="76" t="s">
+        <v>80</v>
+      </c>
+      <c r="E47" s="76"/>
+      <c r="F47" s="76"/>
+      <c r="G47" s="76"/>
+      <c r="H47" s="76"/>
+      <c r="I47" s="76"/>
+    </row>
+    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B48" s="76" t="s">
+        <v>326</v>
+      </c>
+      <c r="C48" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="D48" s="76" t="s">
+        <v>81</v>
+      </c>
+      <c r="E48" s="76"/>
+      <c r="F48" s="76"/>
+      <c r="G48" s="76"/>
+      <c r="H48" s="76"/>
+      <c r="I48" s="76"/>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B49" s="76"/>
+      <c r="C49" s="76"/>
+      <c r="D49" s="76"/>
+      <c r="E49" s="76"/>
+      <c r="F49" s="76"/>
+      <c r="G49" s="76"/>
+      <c r="H49" s="76"/>
+      <c r="I49" s="76"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B50" s="76"/>
+      <c r="C50" s="76"/>
+      <c r="D50" s="76"/>
+      <c r="E50" s="76"/>
+      <c r="F50" s="76"/>
+      <c r="G50" s="76"/>
+      <c r="H50" s="76"/>
+      <c r="I50" s="76"/>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A51" s="76"/>
+      <c r="B51" s="76" t="s">
+        <v>327</v>
+      </c>
+      <c r="C51" s="76"/>
+      <c r="D51" s="76"/>
+      <c r="E51" s="76"/>
+      <c r="F51" s="76"/>
+      <c r="G51" s="76"/>
+      <c r="H51" s="76" t="s">
+        <v>382</v>
+      </c>
+      <c r="I51" s="76"/>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A52" s="76"/>
+      <c r="B52" s="76" t="s">
+        <v>348</v>
+      </c>
+      <c r="C52" s="76"/>
+      <c r="D52" s="76"/>
+      <c r="E52" s="76"/>
+      <c r="F52" s="76"/>
+      <c r="G52" s="76"/>
+      <c r="H52" s="76" t="s">
+        <v>386</v>
+      </c>
+      <c r="I52" s="76"/>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A53" s="76"/>
+      <c r="B53" s="76"/>
+      <c r="C53" s="76"/>
+      <c r="D53" s="76"/>
+      <c r="E53" s="76"/>
+      <c r="F53" s="76"/>
+      <c r="G53" s="76"/>
+      <c r="H53" s="78" t="s">
+        <v>383</v>
+      </c>
+      <c r="I53" s="76"/>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A54" s="76" t="s">
+        <v>328</v>
+      </c>
+      <c r="B54" s="76" t="s">
+        <v>329</v>
+      </c>
+      <c r="C54" s="76" t="s">
+        <v>347</v>
+      </c>
+      <c r="D54" s="76"/>
+      <c r="E54" s="76"/>
+      <c r="F54" s="76"/>
+      <c r="G54" s="76"/>
+      <c r="H54" s="78" t="s">
+        <v>384</v>
+      </c>
+      <c r="I54" s="76"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A55" s="76"/>
+      <c r="B55" s="76" t="s">
+        <v>375</v>
+      </c>
+      <c r="C55" s="76"/>
+      <c r="D55" s="76"/>
+      <c r="E55" s="76"/>
+      <c r="F55" s="76"/>
+      <c r="G55" s="76"/>
+      <c r="H55" s="78" t="s">
+        <v>385</v>
+      </c>
+      <c r="I55" s="76"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A56" s="91" t="s">
+        <v>390</v>
+      </c>
+      <c r="B56" s="78" t="s">
+        <v>376</v>
+      </c>
+      <c r="C56" s="76"/>
+      <c r="D56" s="76"/>
+      <c r="E56" s="76"/>
+      <c r="F56" s="76"/>
+      <c r="G56" s="76"/>
+      <c r="H56" s="76"/>
+      <c r="I56" s="76"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" s="91" t="s">
+        <v>391</v>
+      </c>
+      <c r="B57" s="78" t="s">
+        <v>388</v>
+      </c>
+      <c r="C57" s="76"/>
+      <c r="D57" s="76"/>
+      <c r="E57" s="76"/>
+      <c r="F57" s="76"/>
+      <c r="G57" s="76"/>
+      <c r="H57" s="76"/>
+      <c r="I57" s="76"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" s="91"/>
+      <c r="B58" s="76" t="s">
+        <v>365</v>
+      </c>
+      <c r="C58" s="76"/>
+      <c r="D58" s="76"/>
+      <c r="E58" s="76"/>
+      <c r="F58" s="76"/>
+      <c r="G58" s="76"/>
+      <c r="H58" s="76" t="s">
+        <v>391</v>
+      </c>
+      <c r="I58" s="76"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" s="91" t="s">
+        <v>392</v>
+      </c>
+      <c r="B59" s="78" t="s">
+        <v>366</v>
+      </c>
+      <c r="C59" s="76"/>
+      <c r="D59" s="76"/>
+      <c r="E59" s="76"/>
+      <c r="F59" s="76"/>
+      <c r="G59" s="76"/>
+      <c r="H59" s="76" t="s">
+        <v>389</v>
+      </c>
+      <c r="I59" s="76"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" s="91" t="s">
+        <v>393</v>
+      </c>
+      <c r="B60" s="78" t="s">
+        <v>394</v>
+      </c>
+      <c r="F60" s="76"/>
+      <c r="G60" s="76"/>
+      <c r="H60" s="76"/>
+      <c r="I60" s="76"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61" s="91"/>
+      <c r="B61" s="78"/>
+      <c r="F61" s="76"/>
+      <c r="G61" s="76"/>
+      <c r="H61" s="76"/>
+      <c r="I61" s="76"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" s="76" t="s">
+        <v>359</v>
+      </c>
+      <c r="B62" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="C62" s="80"/>
+      <c r="D62" s="80"/>
+      <c r="E62" s="76"/>
+      <c r="F62" s="76"/>
+      <c r="H62" s="79" t="s">
+        <v>284</v>
+      </c>
+      <c r="I62" s="80"/>
+      <c r="J62" s="80"/>
+      <c r="L62" s="79" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" s="76" t="s">
+        <v>361</v>
+      </c>
+      <c r="B63" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="C63" s="82" t="s">
+        <v>286</v>
+      </c>
+      <c r="D63" s="82" t="s">
+        <v>251</v>
+      </c>
+      <c r="E63" s="76"/>
+      <c r="F63" s="76"/>
+      <c r="H63" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="I63" s="82" t="s">
+        <v>286</v>
+      </c>
+      <c r="J63" s="82" t="s">
+        <v>251</v>
+      </c>
+      <c r="L63" s="83" t="s">
+        <v>378</v>
+      </c>
+      <c r="M63" s="83" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A64" s="76" t="s">
+        <v>363</v>
+      </c>
+      <c r="B64" s="82" t="s">
+        <v>339</v>
+      </c>
+      <c r="C64" s="82" t="s">
+        <v>340</v>
+      </c>
+      <c r="D64" s="82">
+        <v>1</v>
+      </c>
+      <c r="E64" s="76"/>
+      <c r="F64" s="76"/>
+      <c r="H64" s="82" t="s">
+        <v>339</v>
+      </c>
+      <c r="I64" s="82" t="s">
+        <v>340</v>
+      </c>
+      <c r="J64" s="82">
+        <v>1</v>
+      </c>
+      <c r="L64" s="82" t="s">
+        <v>339</v>
+      </c>
+      <c r="M64" s="82" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A65" s="76" t="s">
+        <v>390</v>
+      </c>
+      <c r="B65" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="C65" s="82" t="s">
+        <v>342</v>
+      </c>
+      <c r="D65" s="82">
+        <v>1</v>
+      </c>
+      <c r="E65" s="76"/>
+      <c r="F65" s="76"/>
+      <c r="H65" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="I65" s="82" t="s">
+        <v>342</v>
+      </c>
+      <c r="J65" s="82">
+        <v>1</v>
+      </c>
+      <c r="L65" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="M65" s="82" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A66" s="76" t="s">
+        <v>392</v>
+      </c>
+      <c r="B66" s="82" t="s">
+        <v>343</v>
+      </c>
+      <c r="C66" s="82" t="s">
+        <v>344</v>
+      </c>
+      <c r="D66" s="82">
+        <v>0</v>
+      </c>
+      <c r="E66" s="76"/>
+      <c r="F66" s="76"/>
+      <c r="H66" s="82" t="s">
+        <v>343</v>
+      </c>
+      <c r="I66" s="82" t="s">
+        <v>344</v>
+      </c>
+      <c r="J66" s="82">
+        <v>0</v>
+      </c>
+      <c r="L66" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="M66" s="82" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A67" s="76"/>
+      <c r="B67" s="82" t="s">
+        <v>345</v>
+      </c>
+      <c r="C67" s="82" t="s">
+        <v>346</v>
+      </c>
+      <c r="D67" s="82">
+        <v>1</v>
+      </c>
+      <c r="E67" s="76"/>
+      <c r="F67" s="76"/>
+      <c r="H67" s="82" t="s">
+        <v>345</v>
+      </c>
+      <c r="I67" s="82" t="s">
+        <v>346</v>
+      </c>
+      <c r="J67" s="82">
+        <v>1</v>
+      </c>
+      <c r="L67" s="82" t="s">
+        <v>343</v>
+      </c>
+      <c r="M67" s="82" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A68" s="76"/>
+      <c r="B68" s="76"/>
+      <c r="C68" s="76"/>
+      <c r="D68" s="76"/>
+      <c r="E68" s="76"/>
+      <c r="F68" s="76"/>
+      <c r="H68" s="76"/>
+      <c r="I68" s="76"/>
+      <c r="J68" s="76"/>
+      <c r="L68" s="82" t="s">
+        <v>345</v>
+      </c>
+      <c r="M68" s="82" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" s="76"/>
+      <c r="B69" s="76"/>
+      <c r="C69" s="76"/>
+      <c r="D69" s="76"/>
+      <c r="E69" s="76"/>
+      <c r="F69" s="76"/>
+      <c r="H69" s="76"/>
+      <c r="I69" s="76"/>
+      <c r="J69" s="76"/>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A70" s="76" t="s">
+        <v>360</v>
+      </c>
+      <c r="B70" s="79" t="s">
+        <v>0</v>
+      </c>
+      <c r="C70" s="80"/>
+      <c r="D70" s="80"/>
+      <c r="E70" s="80" t="s">
+        <v>212</v>
+      </c>
+      <c r="F70" s="76"/>
+      <c r="H70" s="79" t="s">
+        <v>0</v>
+      </c>
+      <c r="I70" s="80"/>
+      <c r="J70" s="80"/>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A71" s="76" t="s">
+        <v>362</v>
+      </c>
+      <c r="B71" s="81" t="s">
+        <v>1</v>
+      </c>
+      <c r="C71" s="82" t="s">
+        <v>2</v>
+      </c>
+      <c r="D71" s="82" t="s">
+        <v>233</v>
+      </c>
+      <c r="E71" s="83" t="s">
+        <v>38</v>
+      </c>
+      <c r="F71" s="76"/>
+      <c r="H71" s="81" t="s">
+        <v>1</v>
+      </c>
+      <c r="I71" s="82" t="s">
+        <v>2</v>
+      </c>
+      <c r="J71" s="82" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A72" s="76" t="s">
+        <v>364</v>
+      </c>
+      <c r="B72" s="82" t="s">
+        <v>330</v>
+      </c>
+      <c r="C72" s="82" t="s">
+        <v>331</v>
+      </c>
+      <c r="D72" s="82" t="s">
+        <v>332</v>
+      </c>
+      <c r="E72" s="82" t="s">
+        <v>339</v>
+      </c>
+      <c r="F72" s="76"/>
+      <c r="H72" s="82" t="s">
+        <v>330</v>
+      </c>
+      <c r="I72" s="82" t="s">
+        <v>331</v>
+      </c>
+      <c r="J72" s="82" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A73" s="76"/>
+      <c r="B73" s="82" t="s">
+        <v>333</v>
+      </c>
+      <c r="C73" s="82" t="s">
+        <v>334</v>
+      </c>
+      <c r="D73" s="82" t="s">
+        <v>335</v>
+      </c>
+      <c r="E73" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="F73" s="76"/>
+      <c r="H73" s="82" t="s">
+        <v>333</v>
+      </c>
+      <c r="I73" s="82" t="s">
+        <v>334</v>
+      </c>
+      <c r="J73" s="82" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A74" s="76"/>
+      <c r="B74" s="82" t="s">
+        <v>336</v>
+      </c>
+      <c r="C74" s="82" t="s">
+        <v>337</v>
+      </c>
+      <c r="D74" s="82" t="s">
+        <v>338</v>
+      </c>
+      <c r="E74" s="82" t="s">
+        <v>341</v>
+      </c>
+      <c r="H74" s="82" t="s">
+        <v>336</v>
+      </c>
+      <c r="I74" s="82" t="s">
+        <v>337</v>
+      </c>
+      <c r="J74" s="82" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B75" s="82" t="s">
+        <v>349</v>
+      </c>
+      <c r="C75" s="82" t="s">
+        <v>350</v>
+      </c>
+      <c r="D75" s="82" t="s">
+        <v>351</v>
+      </c>
+      <c r="E75" s="82" t="s">
+        <v>343</v>
+      </c>
+      <c r="H75" s="82" t="s">
+        <v>349</v>
+      </c>
+      <c r="I75" s="82" t="s">
+        <v>350</v>
+      </c>
+      <c r="J75" s="82" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B76" s="82" t="s">
+        <v>379</v>
+      </c>
+      <c r="C76" s="82" t="s">
+        <v>380</v>
+      </c>
+      <c r="D76" s="82" t="s">
+        <v>381</v>
+      </c>
+      <c r="E76" s="82" t="s">
+        <v>343</v>
+      </c>
+      <c r="I76" s="76"/>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B77" s="76"/>
+      <c r="C77" s="76"/>
+      <c r="D77" s="76"/>
+      <c r="E77" s="76"/>
+      <c r="I77" s="76"/>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B78" s="76"/>
+      <c r="C78" s="76"/>
+      <c r="D78" s="76"/>
+      <c r="E78" s="76"/>
+      <c r="H78" s="75" t="s">
+        <v>395</v>
+      </c>
+      <c r="I78" s="76"/>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A79" s="76" t="s">
+        <v>371</v>
+      </c>
+      <c r="B79" s="79" t="s">
+        <v>16</v>
+      </c>
+      <c r="C79" s="85" t="s">
+        <v>374</v>
+      </c>
+      <c r="D79" s="86"/>
+      <c r="E79" s="76"/>
+      <c r="F79" s="76"/>
+      <c r="G79" s="76"/>
+      <c r="H79" s="76"/>
+      <c r="I79" s="76"/>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A80" s="76" t="s">
+        <v>390</v>
+      </c>
+      <c r="B80" s="87" t="s">
+        <v>373</v>
+      </c>
+      <c r="C80" s="88" t="s">
+        <v>1</v>
+      </c>
+      <c r="D80" s="88" t="s">
+        <v>84</v>
+      </c>
+      <c r="E80" s="82" t="s">
+        <v>3</v>
+      </c>
+      <c r="F80" s="84" t="s">
+        <v>17</v>
+      </c>
+      <c r="G80" s="76"/>
+      <c r="H80" s="79" t="s">
+        <v>13</v>
+      </c>
+      <c r="I80" s="80"/>
+      <c r="J80" s="80" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" s="76" t="s">
+        <v>393</v>
+      </c>
+      <c r="B81" s="82">
+        <v>1</v>
+      </c>
+      <c r="C81" s="82" t="s">
+        <v>330</v>
+      </c>
+      <c r="D81" s="82" t="s">
+        <v>293</v>
+      </c>
+      <c r="E81" s="82">
+        <v>100</v>
+      </c>
+      <c r="F81" s="82">
+        <v>5</v>
+      </c>
+      <c r="G81" s="76"/>
+      <c r="H81" s="81" t="s">
+        <v>283</v>
+      </c>
+      <c r="I81" s="82" t="s">
+        <v>286</v>
+      </c>
+      <c r="J81" s="83" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" s="76"/>
+      <c r="B82" s="82">
+        <v>2</v>
+      </c>
+      <c r="C82" s="82" t="s">
+        <v>330</v>
+      </c>
+      <c r="D82" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="E82" s="82">
+        <v>110</v>
+      </c>
+      <c r="F82" s="82">
+        <v>7</v>
+      </c>
+      <c r="G82" s="76"/>
+      <c r="H82" s="82" t="s">
+        <v>396</v>
+      </c>
+      <c r="I82" s="82" t="s">
+        <v>405</v>
+      </c>
+      <c r="J82" s="82" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="76"/>
+      <c r="B83" s="82">
+        <v>3</v>
+      </c>
+      <c r="C83" s="82" t="s">
+        <v>333</v>
+      </c>
+      <c r="D83" s="82" t="s">
+        <v>293</v>
+      </c>
+      <c r="E83" s="82">
+        <v>120</v>
+      </c>
+      <c r="F83" s="82">
+        <v>0</v>
+      </c>
+      <c r="G83" s="76"/>
+      <c r="H83" s="82" t="s">
+        <v>397</v>
+      </c>
+      <c r="I83" s="82" t="s">
+        <v>406</v>
+      </c>
+      <c r="J83" s="82" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="76"/>
+      <c r="B84" s="82">
+        <v>4</v>
+      </c>
+      <c r="C84" s="82" t="s">
+        <v>333</v>
+      </c>
+      <c r="D84" s="82" t="s">
+        <v>85</v>
+      </c>
+      <c r="E84" s="82">
+        <v>100</v>
+      </c>
+      <c r="F84" s="82">
+        <v>2</v>
+      </c>
+      <c r="G84" s="76"/>
+      <c r="H84" s="82" t="s">
+        <v>398</v>
+      </c>
+      <c r="I84" s="82" t="s">
+        <v>407</v>
+      </c>
+      <c r="J84" s="82" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="76"/>
+      <c r="B85" s="82">
+        <v>5</v>
+      </c>
+      <c r="C85" s="82" t="s">
+        <v>333</v>
+      </c>
+      <c r="D85" s="82" t="s">
+        <v>86</v>
+      </c>
+      <c r="E85" s="82">
+        <v>150</v>
+      </c>
+      <c r="F85" s="82">
+        <v>8</v>
+      </c>
+      <c r="G85" s="76"/>
+      <c r="H85" s="82" t="s">
+        <v>399</v>
+      </c>
+      <c r="I85" s="82" t="s">
+        <v>408</v>
+      </c>
+      <c r="J85" s="82" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="76"/>
+      <c r="B86" s="82">
+        <v>6</v>
+      </c>
+      <c r="C86" s="82" t="s">
+        <v>336</v>
+      </c>
+      <c r="D86" s="82" t="s">
+        <v>293</v>
+      </c>
+      <c r="E86" s="82">
+        <v>120</v>
+      </c>
+      <c r="F86" s="82">
+        <v>9</v>
+      </c>
+      <c r="G86" s="76"/>
+      <c r="H86" s="82" t="s">
+        <v>400</v>
+      </c>
+      <c r="I86" s="82" t="s">
+        <v>409</v>
+      </c>
+      <c r="J86" s="82" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="76"/>
+      <c r="B87" s="76"/>
+      <c r="C87" s="76"/>
+      <c r="D87" s="76"/>
+      <c r="E87" s="76"/>
+      <c r="F87" s="76"/>
+      <c r="G87" s="76"/>
+      <c r="H87" s="82" t="s">
+        <v>401</v>
+      </c>
+      <c r="I87" s="82" t="s">
+        <v>410</v>
+      </c>
+      <c r="J87" s="82" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="76"/>
+      <c r="B88" s="76"/>
+      <c r="C88" s="76"/>
+      <c r="D88" s="76"/>
+      <c r="E88" s="76"/>
+      <c r="F88" s="76"/>
+      <c r="G88" s="76"/>
+      <c r="H88" s="82" t="s">
+        <v>402</v>
+      </c>
+      <c r="I88" s="82" t="s">
+        <v>411</v>
+      </c>
+      <c r="J88" s="82" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="76" t="s">
+        <v>372</v>
+      </c>
+      <c r="B89" s="79" t="s">
+        <v>15</v>
+      </c>
+      <c r="C89" s="89" t="s">
+        <v>212</v>
+      </c>
+      <c r="D89" s="90"/>
+      <c r="E89" s="76"/>
+      <c r="F89" s="76"/>
+      <c r="G89" s="76"/>
+      <c r="H89" s="82" t="s">
+        <v>403</v>
+      </c>
+      <c r="I89" s="82" t="s">
+        <v>412</v>
+      </c>
+      <c r="J89" s="82" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B90" s="81" t="s">
+        <v>9</v>
+      </c>
+      <c r="C90" s="83" t="s">
+        <v>373</v>
+      </c>
+      <c r="D90" s="84" t="s">
+        <v>369</v>
+      </c>
+      <c r="F90" s="76"/>
+      <c r="G90" s="76"/>
+      <c r="H90" s="76"/>
+      <c r="I90" s="76"/>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B91" s="82" t="s">
+        <v>367</v>
+      </c>
+      <c r="C91" s="82">
+        <v>1</v>
+      </c>
+      <c r="D91" s="82">
+        <v>1</v>
+      </c>
+      <c r="F91" s="76"/>
+      <c r="G91" s="76"/>
+      <c r="H91" s="76"/>
+      <c r="I91" s="76"/>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B92" s="82" t="s">
+        <v>367</v>
+      </c>
+      <c r="C92" s="82">
+        <v>2</v>
+      </c>
+      <c r="D92" s="82">
+        <v>2</v>
+      </c>
+      <c r="F92" s="76"/>
+      <c r="G92" s="76"/>
+      <c r="H92" s="76"/>
+      <c r="I92" s="76"/>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B93" s="82" t="s">
+        <v>368</v>
+      </c>
+      <c r="C93" s="82">
+        <v>3</v>
+      </c>
+      <c r="D93" s="82">
+        <v>3</v>
+      </c>
+      <c r="F93" s="76"/>
+      <c r="G93" s="76"/>
+      <c r="H93" s="76"/>
+      <c r="I93" s="76"/>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B94" s="82" t="s">
+        <v>368</v>
+      </c>
+      <c r="C94" s="82">
+        <v>4</v>
+      </c>
+      <c r="D94" s="82">
+        <v>5</v>
+      </c>
+      <c r="F94" s="76"/>
+      <c r="G94" s="76"/>
+      <c r="H94" s="76"/>
+      <c r="I94" s="76"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B95" s="82" t="s">
+        <v>368</v>
+      </c>
+      <c r="C95" s="82">
+        <v>6</v>
+      </c>
+      <c r="D95" s="82">
+        <v>1</v>
+      </c>
+      <c r="F95" s="76"/>
+      <c r="G95" s="76"/>
+      <c r="H95" s="76"/>
+      <c r="I95" s="76"/>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B96" s="82" t="s">
+        <v>370</v>
+      </c>
+      <c r="C96" s="82">
+        <v>6</v>
+      </c>
+      <c r="D96" s="82">
+        <v>1</v>
+      </c>
+      <c r="F96" s="76"/>
+      <c r="G96" s="76"/>
+      <c r="H96" s="76"/>
+      <c r="I96" s="76"/>
+    </row>
+    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B97" s="76"/>
+      <c r="C97" s="76"/>
+      <c r="D97" s="76"/>
+      <c r="E97" s="76"/>
+      <c r="F97" s="76"/>
+      <c r="G97" s="76"/>
+      <c r="H97" s="76"/>
+      <c r="I97" s="76"/>
+    </row>
+    <row r="98" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B98" s="76"/>
+      <c r="C98" s="76"/>
+      <c r="D98" s="76"/>
+      <c r="E98" s="76"/>
+      <c r="F98" s="76"/>
+      <c r="G98" s="76"/>
+      <c r="H98" s="76"/>
+      <c r="I98" s="76"/>
+    </row>
+    <row r="99" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B99" s="76"/>
+      <c r="C99" s="76"/>
+      <c r="D99" s="76"/>
+      <c r="E99" s="76"/>
+      <c r="F99" s="76"/>
+      <c r="G99" s="76"/>
+      <c r="H99" s="76"/>
+      <c r="I99" s="76"/>
+    </row>
+    <row r="100" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B100" s="76"/>
+      <c r="C100" s="76"/>
+      <c r="D100" s="76"/>
+      <c r="E100" s="76"/>
+      <c r="F100" s="76"/>
+      <c r="G100" s="76"/>
+      <c r="H100" s="76"/>
+      <c r="I100" s="76"/>
+    </row>
+    <row r="101" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B101" s="76"/>
+      <c r="C101" s="76"/>
+      <c r="D101" s="76"/>
+      <c r="E101" s="76"/>
+      <c r="F101" s="76"/>
+      <c r="G101" s="76"/>
+      <c r="H101" s="76"/>
+      <c r="I101" s="76"/>
+    </row>
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B102" s="76"/>
+      <c r="C102" s="76"/>
+      <c r="D102" s="76"/>
+      <c r="E102" s="76"/>
+      <c r="F102" s="76"/>
+      <c r="G102" s="76"/>
+      <c r="H102" s="76"/>
+      <c r="I102" s="76"/>
+    </row>
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B103" s="76"/>
+      <c r="C103" s="76"/>
+      <c r="D103" s="76"/>
+      <c r="E103" s="76"/>
+      <c r="F103" s="76"/>
+      <c r="G103" s="76"/>
+      <c r="H103" s="76"/>
+      <c r="I103" s="76"/>
+    </row>
+    <row r="104" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B104" s="76"/>
+      <c r="C104" s="76"/>
+      <c r="D104" s="76"/>
+      <c r="E104" s="76"/>
+      <c r="F104" s="76"/>
+      <c r="G104" s="76"/>
+      <c r="H104" s="76"/>
+      <c r="I104" s="76"/>
+    </row>
+    <row r="105" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B105" s="76"/>
+      <c r="C105" s="76"/>
+      <c r="D105" s="76"/>
+      <c r="E105" s="76"/>
+      <c r="F105" s="76"/>
+      <c r="G105" s="76"/>
+      <c r="H105" s="76"/>
+      <c r="I105" s="76"/>
+    </row>
+    <row r="106" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B106" s="76"/>
+      <c r="C106" s="76"/>
+      <c r="D106" s="76"/>
+      <c r="E106" s="76"/>
+      <c r="F106" s="76"/>
+      <c r="G106" s="76"/>
+      <c r="H106" s="76"/>
+      <c r="I106" s="76"/>
+    </row>
+    <row r="107" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B107" s="76"/>
+      <c r="C107" s="76"/>
+      <c r="D107" s="76"/>
+      <c r="E107" s="76"/>
+      <c r="F107" s="76"/>
+      <c r="G107" s="76"/>
+      <c r="H107" s="76"/>
+      <c r="I107" s="76"/>
+    </row>
+    <row r="108" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B108" s="76"/>
+      <c r="C108" s="76"/>
+      <c r="D108" s="76"/>
+      <c r="E108" s="76"/>
+      <c r="F108" s="76"/>
+      <c r="G108" s="76"/>
+      <c r="H108" s="76"/>
+      <c r="I108" s="76"/>
+    </row>
+    <row r="109" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B109" s="76"/>
+      <c r="C109" s="76"/>
+      <c r="D109" s="76"/>
+      <c r="E109" s="76"/>
+      <c r="F109" s="76"/>
+      <c r="G109" s="76"/>
+      <c r="H109" s="76"/>
+      <c r="I109" s="76"/>
+    </row>
+    <row r="110" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B110" s="76"/>
+      <c r="C110" s="76"/>
+      <c r="D110" s="76"/>
+      <c r="E110" s="76"/>
+      <c r="F110" s="76"/>
+      <c r="G110" s="76"/>
+      <c r="H110" s="76"/>
+      <c r="I110" s="76"/>
+    </row>
+    <row r="111" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B111" s="76"/>
+      <c r="C111" s="76"/>
+      <c r="D111" s="76"/>
+      <c r="E111" s="76"/>
+      <c r="F111" s="76"/>
+      <c r="G111" s="76"/>
+      <c r="H111" s="76"/>
+      <c r="I111" s="76"/>
+    </row>
+    <row r="112" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B112" s="76"/>
+      <c r="C112" s="76"/>
+      <c r="D112" s="76"/>
+      <c r="E112" s="76"/>
+      <c r="F112" s="76"/>
+      <c r="G112" s="76"/>
+      <c r="H112" s="76"/>
+      <c r="I112" s="76"/>
+    </row>
+    <row r="113" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B113" s="76"/>
+      <c r="C113" s="76"/>
+      <c r="D113" s="76"/>
+      <c r="E113" s="76"/>
+      <c r="F113" s="76"/>
+      <c r="G113" s="76"/>
+      <c r="H113" s="76"/>
+      <c r="I113" s="76"/>
+    </row>
+    <row r="114" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B114" s="76"/>
+      <c r="C114" s="76"/>
+      <c r="D114" s="76"/>
+      <c r="E114" s="76"/>
+      <c r="F114" s="76"/>
+      <c r="G114" s="76"/>
+      <c r="H114" s="76"/>
+      <c r="I114" s="76"/>
+    </row>
+    <row r="115" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B115" s="76"/>
+      <c r="C115" s="76"/>
+      <c r="D115" s="76"/>
+      <c r="E115" s="76"/>
+      <c r="F115" s="76"/>
+      <c r="G115" s="76"/>
+      <c r="H115" s="76"/>
+      <c r="I115" s="76"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C79:D79"/>
+  </mergeCells>
+  <phoneticPr fontId="30" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A2:U43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3479,12 +6295,12 @@
       <c r="Q13" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="R13" s="64" t="s">
+      <c r="R13" s="65" t="s">
         <v>68</v>
       </c>
-      <c r="S13" s="64"/>
-      <c r="T13" s="64"/>
-      <c r="U13" s="64"/>
+      <c r="S13" s="65"/>
+      <c r="T13" s="65"/>
+      <c r="U13" s="65"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="D14" s="5"/>
@@ -3497,10 +6313,10 @@
       <c r="Q14" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="R14" s="64"/>
-      <c r="S14" s="64"/>
-      <c r="T14" s="64"/>
-      <c r="U14" s="64"/>
+      <c r="R14" s="65"/>
+      <c r="S14" s="65"/>
+      <c r="T14" s="65"/>
+      <c r="U14" s="65"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
@@ -3799,7 +6615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A2:AJ77"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4075,10 +6891,10 @@
       <c r="W18" s="5"/>
     </row>
     <row r="19" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="P19" s="69" t="s">
+      <c r="P19" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="Q19" s="69"/>
+      <c r="Q19" s="70"/>
       <c r="T19" s="4" t="s">
         <v>9</v>
       </c>
@@ -4096,10 +6912,10 @@
       <c r="P20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="Q20" s="68" t="s">
+      <c r="Q20" s="69" t="s">
         <v>14</v>
       </c>
-      <c r="R20" s="68"/>
+      <c r="R20" s="69"/>
       <c r="T20" s="4" t="s">
         <v>94</v>
       </c>
@@ -4117,10 +6933,10 @@
       <c r="P21" s="4">
         <v>1</v>
       </c>
-      <c r="Q21" s="68" t="s">
+      <c r="Q21" s="69" t="s">
         <v>99</v>
       </c>
-      <c r="R21" s="68"/>
+      <c r="R21" s="69"/>
       <c r="T21" s="4" t="s">
         <v>94</v>
       </c>
@@ -4138,10 +6954,10 @@
       <c r="P22" s="4">
         <v>2</v>
       </c>
-      <c r="Q22" s="68" t="s">
+      <c r="Q22" s="69" t="s">
         <v>100</v>
       </c>
-      <c r="R22" s="68"/>
+      <c r="R22" s="69"/>
       <c r="T22" s="4" t="s">
         <v>94</v>
       </c>
@@ -4159,10 +6975,10 @@
       <c r="P23" s="4">
         <v>3</v>
       </c>
-      <c r="Q23" s="68" t="s">
+      <c r="Q23" s="69" t="s">
         <v>101</v>
       </c>
-      <c r="R23" s="68"/>
+      <c r="R23" s="69"/>
       <c r="T23" s="4"/>
       <c r="U23" s="4"/>
       <c r="V23" s="4"/>
@@ -4181,10 +6997,10 @@
       <c r="P24" s="4">
         <v>4</v>
       </c>
-      <c r="Q24" s="68" t="s">
+      <c r="Q24" s="69" t="s">
         <v>102</v>
       </c>
-      <c r="R24" s="68"/>
+      <c r="R24" s="69"/>
       <c r="T24" s="4" t="s">
         <v>95</v>
       </c>
@@ -4829,16 +7645,16 @@
       </c>
     </row>
     <row r="48" spans="3:36" x14ac:dyDescent="0.25">
-      <c r="C48" s="65" t="s">
+      <c r="C48" s="66" t="s">
         <v>220</v>
       </c>
-      <c r="D48" s="66"/>
-      <c r="E48" s="66"/>
-      <c r="F48" s="66"/>
-      <c r="G48" s="66"/>
-      <c r="H48" s="66"/>
-      <c r="I48" s="66"/>
-      <c r="J48" s="66"/>
+      <c r="D48" s="67"/>
+      <c r="E48" s="67"/>
+      <c r="F48" s="67"/>
+      <c r="G48" s="67"/>
+      <c r="H48" s="67"/>
+      <c r="I48" s="67"/>
+      <c r="J48" s="67"/>
       <c r="O48" s="29">
         <v>3</v>
       </c>
@@ -4868,16 +7684,16 @@
       </c>
     </row>
     <row r="49" spans="3:32" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C49" s="67" t="s">
+      <c r="C49" s="68" t="s">
         <v>219</v>
       </c>
-      <c r="D49" s="67"/>
-      <c r="E49" s="67"/>
-      <c r="F49" s="67"/>
-      <c r="G49" s="67"/>
-      <c r="H49" s="67"/>
-      <c r="I49" s="67"/>
-      <c r="J49" s="67"/>
+      <c r="D49" s="68"/>
+      <c r="E49" s="68"/>
+      <c r="F49" s="68"/>
+      <c r="G49" s="68"/>
+      <c r="H49" s="68"/>
+      <c r="I49" s="68"/>
+      <c r="J49" s="68"/>
       <c r="O49" s="29">
         <v>4</v>
       </c>
@@ -5332,7 +8148,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:N26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
lesson16-database hoan thanh database
</commit_message>
<xml_diff>
--- a/Java25 Quyen Phan Database Design.xlsx
+++ b/Java25 Quyen Phan Database Design.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qphan\Desktop\bkit\course - webapp\java25\3. Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D451E773-E33C-415A-860A-3D0FE299A19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BCB4CA4-FEDD-49AF-946C-60B105CDE768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="588" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1860" windowWidth="38640" windowHeight="21120" tabRatio="588" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Mô hình quan niệm" sheetId="1" r:id="rId1"/>
@@ -520,7 +520,247 @@
     <author>Quyen Ngoc Phan</author>
   </authors>
   <commentList>
-    <comment ref="D63" authorId="0" shapeId="0" xr:uid="{637B7D0C-5A9B-4DE9-9EE9-44588ADC702A}">
+    <comment ref="M6" authorId="0" shapeId="0" xr:uid="{01E74519-0E51-4163-9248-3733724A61CA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Chi tiết nhập hàng cho mặt hàng để quản lý lịch sử giá mua</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B9" authorId="0" shapeId="0" xr:uid="{874A984F-D2B7-4D49-BCF6-0718734568A4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Thuộc tính dẫn xuất</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C9" authorId="0" shapeId="0" xr:uid="{30C09ED4-25E6-4906-BB92-CFFDC2539127}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+0/1 active || inactive</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0" xr:uid="{F5C6CDFA-44AD-4334-8D13-2296170C573D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Chất liệu</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O10" authorId="0" shapeId="0" xr:uid="{37A6BE56-4EBA-4081-9A2F-AA7326C00113}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Thời gian cập nhật trạng thái đơn hàng</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G11" authorId="0" shapeId="0" xr:uid="{271AEF69-95D0-462A-A025-5DFC63B11267}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dmy hms</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M11" authorId="0" shapeId="0" xr:uid="{09E5306D-6BE9-4201-A5F8-3A1C83E6CE46}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+d/m/y h:m:s</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0" xr:uid="{6C563392-045E-4C1D-9208-98CD2ABE144A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+nullable</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G12" authorId="0" shapeId="0" xr:uid="{A79DEE70-C39A-4DC4-B198-E9B63B7D0B2B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+dmy</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{711549CA-335B-4941-92E0-74FB3628E974}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Quyen Ngoc Phan:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+nullable</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D65" authorId="0" shapeId="0" xr:uid="{637B7D0C-5A9B-4DE9-9EE9-44588ADC702A}">
       <text>
         <r>
           <rPr>
@@ -544,7 +784,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J63" authorId="0" shapeId="0" xr:uid="{E2760732-53B2-4D5A-92BC-1214FC620FFD}">
+    <comment ref="K65" authorId="0" shapeId="0" xr:uid="{E2760732-53B2-4D5A-92BC-1214FC620FFD}">
       <text>
         <r>
           <rPr>
@@ -568,7 +808,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J81" authorId="0" shapeId="0" xr:uid="{376EF730-7F42-4051-8140-510111B257ED}">
+    <comment ref="K83" authorId="0" shapeId="0" xr:uid="{376EF730-7F42-4051-8140-510111B257ED}">
       <text>
         <r>
           <rPr>
@@ -597,7 +837,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="703" uniqueCount="347">
   <si>
     <t>MatHang</t>
   </si>
@@ -1711,12 +1951,264 @@
   <si>
     <t>C02_STATUS</t>
   </si>
+  <si>
+    <t>T04_SIZE</t>
+  </si>
+  <si>
+    <t>Chú thích</t>
+  </si>
+  <si>
+    <t>C04_SIZE_ID</t>
+  </si>
+  <si>
+    <t>C04_SIZE_NAME</t>
+  </si>
+  <si>
+    <t>C04_GENDER</t>
+  </si>
+  <si>
+    <t>C04_SIZE_DESC</t>
+  </si>
+  <si>
+    <t>T14_ITEM_DETAIL</t>
+  </si>
+  <si>
+    <t>C14_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C14_SIZE_ID</t>
+  </si>
+  <si>
+    <t>C14_SALES_PRICE</t>
+  </si>
+  <si>
+    <t>C14_AMOUNT</t>
+  </si>
+  <si>
+    <t>T05_PROVIDER</t>
+  </si>
+  <si>
+    <t>C05_PROVIDER_ID</t>
+  </si>
+  <si>
+    <t>C05_PROVIDER_NAME</t>
+  </si>
+  <si>
+    <t>C05_PROVIDER_TAX</t>
+  </si>
+  <si>
+    <t>C15_AMOUNT</t>
+  </si>
+  <si>
+    <t>C15_BUY_PRICE</t>
+  </si>
+  <si>
+    <t>T15_ITEM_RECEIPT_DETAIL</t>
+  </si>
+  <si>
+    <t>C15_RECEIPT_DATE</t>
+  </si>
+  <si>
+    <t>Tạo 1 TRIGGER cho T15_ITEM_RECEIPT_DATE</t>
+  </si>
+  <si>
+    <t>- Khi nhập hàng, item sẽ có giá mua mới</t>
+  </si>
+  <si>
+    <t>- Cần cập nhật giá mua mới đó vào C01_BUY_PRICE (thuộc tính dẫn xuất từ ITEM và newest BUY_PRICE ở T15)</t>
+  </si>
+  <si>
+    <t>C01_BUY_PRICE</t>
+  </si>
+  <si>
+    <t>C15_PROVIDER_ID</t>
+  </si>
+  <si>
+    <t>C15_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C01_MATERIAL</t>
+  </si>
+  <si>
+    <t>C01_COLOR</t>
+  </si>
+  <si>
+    <t>Xử lý chỗ MatHang: chất liệu &amp; màu sắc</t>
+  </si>
+  <si>
+    <t>MatHang có ChatLieu|MauSac khác nhau thì xem như là MatHang khác nhau</t>
+  </si>
+  <si>
+    <t>Xử lý cho MatHang: hình ảnh</t>
+  </si>
+  <si>
+    <t>MatHang có thể có nhiều hình ảnh</t>
+  </si>
+  <si>
+    <t>==&gt; Tạo ra một bảng N/N là sự kết hợp giữa MatHang(Table) và HinhAnh(Column)</t>
+  </si>
+  <si>
+    <t>T10_GALLERY</t>
+  </si>
+  <si>
+    <t>C10_ITEM_ID</t>
+  </si>
+  <si>
+    <t>C10_IMAGE_PATH</t>
+  </si>
+  <si>
+    <t>✅</t>
+  </si>
+  <si>
+    <t>⛔</t>
+  </si>
+  <si>
+    <t>T08_CUSTOMER</t>
+  </si>
+  <si>
+    <t>T09_EMPLOYEE</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_NAME</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_EMAIL</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_PHONE</t>
+  </si>
+  <si>
+    <t>C08_SOCIAL_MEDIA</t>
+  </si>
+  <si>
+    <t>C08_SM_TOKEN</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_ADDRESS</t>
+  </si>
+  <si>
+    <t>C08_CUSTOMER_PASSWORD</t>
+  </si>
+  <si>
+    <t>C09_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>C09_EMPLOYEE_NAME</t>
+  </si>
+  <si>
+    <t>C09_EMPLOYEE_EMAIL</t>
+  </si>
+  <si>
+    <t>C09_EMPLOYEE_PHONE</t>
+  </si>
+  <si>
+    <t>T06_ORDER</t>
+  </si>
+  <si>
+    <t>C06_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C06_CUSTOMER_ID</t>
+  </si>
+  <si>
+    <t>C06_DELIVERY_ADDRESS</t>
+  </si>
+  <si>
+    <t>C06_RECEIVER_PHONE</t>
+  </si>
+  <si>
+    <t>C06_ORDER_DATE</t>
+  </si>
+  <si>
+    <t>C06_EXPECTED_DELIVERY_DATE</t>
+  </si>
+  <si>
+    <t>T16_ORDER_DETAIL</t>
+  </si>
+  <si>
+    <t>C16_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C16_AMOUNT</t>
+  </si>
+  <si>
+    <t>C14_ITEM_DETAIL_ID</t>
+  </si>
+  <si>
+    <t>C16_ITEM_DETAIL_ID</t>
+  </si>
+  <si>
+    <t>PK FK</t>
+  </si>
+  <si>
+    <t>C06_DELIVERY_FEE</t>
+  </si>
+  <si>
+    <t>T07_BILL</t>
+  </si>
+  <si>
+    <t>C07_BILL_ID</t>
+  </si>
+  <si>
+    <t>C07_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C10_TOTAL_OF_MONEY</t>
+  </si>
+  <si>
+    <t>T90_PAYMENT_METHOD</t>
+  </si>
+  <si>
+    <t>C90_PAYMENT_METHOD_ID</t>
+  </si>
+  <si>
+    <t>C90_PAYMENT_METHOD_NAME</t>
+  </si>
+  <si>
+    <t>C06_PAYMENT_METHOD_ID</t>
+  </si>
+  <si>
+    <t>T91_ORDER_STATUS</t>
+  </si>
+  <si>
+    <t>C91_ORDER_STATUS_ID</t>
+  </si>
+  <si>
+    <t>C91_ORDER_STATUS_DESC</t>
+  </si>
+  <si>
+    <t>T17_ORDER_STATUS_DETAIL</t>
+  </si>
+  <si>
+    <t>C17_LAST_UPDATED</t>
+  </si>
+  <si>
+    <t>C17_ORDER_ID</t>
+  </si>
+  <si>
+    <t>C17_ORDER_STATUS_ID</t>
+  </si>
+  <si>
+    <t>C17_EMPLOYEE_ID</t>
+  </si>
+  <si>
+    <t>VIEW</t>
+  </si>
+  <si>
+    <t>TRIGGER</t>
+  </si>
+  <si>
+    <t>FUNCTION/PROCEDURE</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="33" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1908,6 +2400,48 @@
       <u/>
       <sz val="10"/>
       <color rgb="FFC00000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="4" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -2137,12 +2671,6 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2173,56 +2701,62 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="16" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3527,14 +4061,52 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D2" s="26" t="s">
-        <v>64</v>
+      <c r="B2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="C2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="D2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="E2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="F2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="G2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="H2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="I2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="J2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="K2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="L2" s="60" t="s">
+        <v>298</v>
+      </c>
+      <c r="M2" s="61" t="s">
+        <v>299</v>
+      </c>
+      <c r="N2" s="61" t="s">
+        <v>299</v>
+      </c>
+      <c r="O2" s="60" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F3" s="9" t="s">
-        <v>117</v>
-      </c>
+      <c r="D3" s="9"/>
+      <c r="F3" s="9"/>
       <c r="J3" s="9" t="s">
         <v>115</v>
       </c>
@@ -4381,10 +4953,10 @@
       <c r="I53" s="27"/>
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A54" s="42" t="s">
+      <c r="A54" s="40" t="s">
         <v>132</v>
       </c>
-      <c r="B54" s="42" t="s">
+      <c r="B54" s="40" t="s">
         <v>133</v>
       </c>
       <c r="C54" s="27" t="s">
@@ -4898,10 +5470,10 @@
       <c r="B79" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C79" s="40" t="s">
+      <c r="C79" s="55" t="s">
         <v>178</v>
       </c>
-      <c r="D79" s="41"/>
+      <c r="D79" s="56"/>
       <c r="E79" s="27"/>
       <c r="F79" s="27"/>
       <c r="G79" s="27"/>
@@ -5282,10 +5854,10 @@
       <c r="I97" s="27"/>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A98" s="48" t="s">
+      <c r="A98" s="46" t="s">
         <v>218</v>
       </c>
-      <c r="B98" s="42" t="s">
+      <c r="B98" s="40" t="s">
         <v>219</v>
       </c>
       <c r="C98" s="27" t="s">
@@ -5344,7 +5916,7 @@
       <c r="I102" s="27"/>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B103" s="47" t="s">
+      <c r="B103" s="45" t="s">
         <v>235</v>
       </c>
       <c r="F103" s="27"/>
@@ -5354,14 +5926,14 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="F104" s="27"/>
-      <c r="G104" s="43" t="s">
+      <c r="G104" s="41" t="s">
         <v>239</v>
       </c>
       <c r="H104" s="27"/>
       <c r="I104" s="27"/>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B105" s="43" t="s">
+      <c r="B105" s="41" t="s">
         <v>8</v>
       </c>
       <c r="C105" s="27"/>
@@ -5460,7 +6032,7 @@
       <c r="B110" s="33" t="s">
         <v>223</v>
       </c>
-      <c r="C110" s="44" t="s">
+      <c r="C110" s="42" t="s">
         <v>228</v>
       </c>
       <c r="D110" s="33" t="s">
@@ -5493,12 +6065,12 @@
       <c r="I112" s="27"/>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B113" s="43" t="s">
+      <c r="B113" s="41" t="s">
         <v>17</v>
       </c>
       <c r="C113" s="27"/>
       <c r="D113" s="27"/>
-      <c r="E113" s="46" t="s">
+      <c r="E113" s="44" t="s">
         <v>233</v>
       </c>
       <c r="F113" s="27"/>
@@ -5528,10 +6100,10 @@
       <c r="B115" s="33" t="s">
         <v>229</v>
       </c>
-      <c r="C115" s="45">
+      <c r="C115" s="43">
         <v>22000</v>
       </c>
-      <c r="D115" s="45">
+      <c r="D115" s="43">
         <v>100000</v>
       </c>
       <c r="E115" s="33" t="s">
@@ -5546,10 +6118,10 @@
       <c r="B116" s="33" t="s">
         <v>230</v>
       </c>
-      <c r="C116" s="45">
+      <c r="C116" s="43">
         <v>50000</v>
       </c>
-      <c r="D116" s="45">
+      <c r="D116" s="43">
         <v>220000</v>
       </c>
       <c r="E116" s="33" t="s">
@@ -5563,7 +6135,7 @@
       <c r="C117" s="33">
         <v>0</v>
       </c>
-      <c r="D117" s="45">
+      <c r="D117" s="43">
         <v>320000</v>
       </c>
       <c r="E117" s="33" t="s">
@@ -5581,10 +6153,10 @@
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A122" s="48" t="s">
+      <c r="A122" s="46" t="s">
         <v>242</v>
       </c>
-      <c r="B122" s="48" t="s">
+      <c r="B122" s="46" t="s">
         <v>243</v>
       </c>
       <c r="C122" s="26" t="s">
@@ -5603,22 +6175,22 @@
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B124" s="47" t="s">
+      <c r="B124" s="45" t="s">
         <v>247</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B125" s="47" t="s">
+      <c r="B125" s="45" t="s">
         <v>248</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B126" s="47" t="s">
+      <c r="B126" s="45" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B129" s="43" t="s">
+      <c r="B129" s="41" t="s">
         <v>8</v>
       </c>
       <c r="C129" s="27"/>
@@ -5672,7 +6244,7 @@
       <c r="B134" s="33" t="s">
         <v>223</v>
       </c>
-      <c r="C134" s="44" t="s">
+      <c r="C134" s="42" t="s">
         <v>228</v>
       </c>
       <c r="D134" s="33" t="s">
@@ -5772,15 +6344,15 @@
       </c>
     </row>
     <row r="146" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B146" s="43" t="s">
+      <c r="B146" s="41" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="147" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B147" s="49" t="s">
+      <c r="B147" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C147" s="49" t="s">
+      <c r="C147" s="47" t="s">
         <v>1</v>
       </c>
       <c r="D147" s="33" t="s">
@@ -5855,2404 +6427,1203 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3F085D2-AFEE-4EB0-86FC-5726E17CEA88}">
-  <dimension ref="A3:P152"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A2:Q154"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" style="26" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" style="26" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" style="26" customWidth="1"/>
-    <col min="4" max="4" width="22.42578125" style="26" customWidth="1"/>
-    <col min="5" max="5" width="20.7109375" style="26" customWidth="1"/>
-    <col min="6" max="6" width="22.7109375" style="26" customWidth="1"/>
-    <col min="7" max="17" width="20.7109375" style="26" customWidth="1"/>
-    <col min="18" max="21" width="12.7109375" style="26" customWidth="1"/>
-    <col min="22" max="16384" width="9.140625" style="26"/>
+    <col min="1" max="1" width="14.7109375" style="27" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="27" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" style="27" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" style="27" customWidth="1"/>
+    <col min="5" max="5" width="20.7109375" style="27" customWidth="1"/>
+    <col min="6" max="6" width="22.7109375" style="27" customWidth="1"/>
+    <col min="7" max="8" width="29.7109375" style="27" customWidth="1"/>
+    <col min="9" max="9" width="27" style="27" customWidth="1"/>
+    <col min="10" max="10" width="25" style="27" customWidth="1"/>
+    <col min="11" max="12" width="20.7109375" style="27" customWidth="1"/>
+    <col min="13" max="13" width="26.28515625" style="27" customWidth="1"/>
+    <col min="14" max="14" width="24.42578125" style="27" customWidth="1"/>
+    <col min="15" max="15" width="26.85546875" style="27" customWidth="1"/>
+    <col min="16" max="16" width="36.5703125" style="27" customWidth="1"/>
+    <col min="17" max="17" width="29.140625" style="27" customWidth="1"/>
+    <col min="18" max="18" width="20.7109375" style="27" customWidth="1"/>
+    <col min="19" max="22" width="12.7109375" style="27" customWidth="1"/>
+    <col min="23" max="16384" width="9.140625" style="27"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-    </row>
-    <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="1" t="s">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B3" s="32" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" s="62" t="s">
+        <v>178</v>
+      </c>
+      <c r="E3" s="63" t="s">
+        <v>326</v>
+      </c>
+      <c r="F3" s="31"/>
+      <c r="K3" s="31"/>
+      <c r="L3" s="31"/>
+      <c r="M3" s="31"/>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="31"/>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="F5" s="31"/>
+      <c r="K5" s="31"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="31"/>
+    </row>
+    <row r="6" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="64" t="s">
         <v>250</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C6" s="64" t="s">
         <v>253</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D6" s="64" t="s">
         <v>254</v>
       </c>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-    </row>
-    <row r="5" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="32" t="s">
+      <c r="E6" s="64" t="s">
+        <v>263</v>
+      </c>
+      <c r="F6" s="64" t="s">
+        <v>274</v>
+      </c>
+      <c r="G6" s="64" t="s">
+        <v>314</v>
+      </c>
+      <c r="H6" s="64" t="s">
+        <v>328</v>
+      </c>
+      <c r="I6" s="64" t="s">
+        <v>300</v>
+      </c>
+      <c r="J6" s="64" t="s">
+        <v>301</v>
+      </c>
+      <c r="K6" s="64" t="s">
+        <v>295</v>
+      </c>
+      <c r="L6" s="64" t="s">
+        <v>269</v>
+      </c>
+      <c r="M6" s="64" t="s">
+        <v>280</v>
+      </c>
+      <c r="N6" s="64" t="s">
+        <v>321</v>
+      </c>
+      <c r="O6" s="64" t="s">
+        <v>339</v>
+      </c>
+      <c r="P6" s="64" t="s">
+        <v>332</v>
+      </c>
+      <c r="Q6" s="64" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="32" t="s">
         <v>251</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C7" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D7" s="32" t="s">
         <v>257</v>
       </c>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
+      <c r="E7" s="32" t="s">
+        <v>265</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>275</v>
+      </c>
+      <c r="G7" s="32" t="s">
+        <v>315</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>329</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>302</v>
+      </c>
+      <c r="J7" s="32" t="s">
+        <v>310</v>
+      </c>
+      <c r="K7" s="32" t="s">
+        <v>296</v>
+      </c>
+      <c r="L7" s="32" t="s">
+        <v>324</v>
+      </c>
+      <c r="M7" s="63" t="s">
+        <v>286</v>
+      </c>
+      <c r="N7" s="63" t="s">
+        <v>322</v>
+      </c>
+      <c r="O7" s="63" t="s">
+        <v>341</v>
+      </c>
+      <c r="P7" s="32" t="s">
+        <v>333</v>
+      </c>
+      <c r="Q7" s="32" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="35" t="s">
         <v>252</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C8" s="35" t="s">
         <v>256</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D8" s="35" t="s">
         <v>258</v>
       </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-    </row>
-    <row r="7" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="34" t="s">
+      <c r="E8" s="62" t="s">
+        <v>266</v>
+      </c>
+      <c r="F8" s="35" t="s">
+        <v>276</v>
+      </c>
+      <c r="G8" s="35" t="s">
+        <v>317</v>
+      </c>
+      <c r="H8" s="34" t="s">
+        <v>330</v>
+      </c>
+      <c r="I8" s="35" t="s">
+        <v>303</v>
+      </c>
+      <c r="J8" s="35" t="s">
+        <v>311</v>
+      </c>
+      <c r="K8" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="L8" s="65" t="s">
+        <v>270</v>
+      </c>
+      <c r="M8" s="63" t="s">
+        <v>287</v>
+      </c>
+      <c r="N8" s="63" t="s">
+        <v>325</v>
+      </c>
+      <c r="O8" s="63" t="s">
+        <v>342</v>
+      </c>
+      <c r="P8" s="62" t="s">
+        <v>334</v>
+      </c>
+      <c r="Q8" s="62" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="35" t="s">
+        <v>285</v>
+      </c>
+      <c r="C9" s="35" t="s">
+        <v>262</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>261</v>
+      </c>
+      <c r="E9" s="62" t="s">
+        <v>267</v>
+      </c>
+      <c r="F9" s="35" t="s">
+        <v>277</v>
+      </c>
+      <c r="G9" s="31" t="s">
+        <v>327</v>
+      </c>
+      <c r="H9" s="35" t="s">
+        <v>331</v>
+      </c>
+      <c r="I9" s="62" t="s">
+        <v>304</v>
+      </c>
+      <c r="J9" s="62" t="s">
+        <v>312</v>
+      </c>
+      <c r="K9" s="35"/>
+      <c r="L9" s="65" t="s">
+        <v>271</v>
+      </c>
+      <c r="M9" s="35" t="s">
+        <v>279</v>
+      </c>
+      <c r="N9" s="35" t="s">
+        <v>323</v>
+      </c>
+      <c r="O9" s="34" t="s">
+        <v>343</v>
+      </c>
+      <c r="P9" s="35"/>
+      <c r="Q9" s="35"/>
+    </row>
+    <row r="10" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="31"/>
+      <c r="B10" s="35" t="s">
+        <v>288</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35" t="s">
+        <v>268</v>
+      </c>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35" t="s">
+        <v>318</v>
+      </c>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35" t="s">
+        <v>305</v>
+      </c>
+      <c r="J10" s="35" t="s">
+        <v>313</v>
+      </c>
+      <c r="K10" s="35"/>
+      <c r="L10" s="35" t="s">
+        <v>272</v>
+      </c>
+      <c r="M10" s="35" t="s">
+        <v>278</v>
+      </c>
+      <c r="N10" s="35"/>
+      <c r="O10" s="35" t="s">
+        <v>340</v>
+      </c>
+      <c r="P10" s="35"/>
+      <c r="Q10" s="35"/>
+    </row>
+    <row r="11" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="35" t="s">
+        <v>289</v>
+      </c>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35" t="s">
+        <v>319</v>
+      </c>
+      <c r="H11" s="35"/>
+      <c r="I11" s="35" t="s">
+        <v>308</v>
+      </c>
+      <c r="J11" s="35"/>
+      <c r="K11" s="35"/>
+      <c r="L11" s="35" t="s">
+        <v>273</v>
+      </c>
+      <c r="M11" s="35" t="s">
+        <v>281</v>
+      </c>
+      <c r="N11" s="35"/>
+      <c r="O11" s="35"/>
+      <c r="P11" s="35"/>
+      <c r="Q11" s="35"/>
+    </row>
+    <row r="12" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="34" t="s">
         <v>260</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="D7" s="34" t="s">
-        <v>261</v>
-      </c>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-      <c r="B8" s="34" t="s">
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35" t="s">
+        <v>320</v>
+      </c>
+      <c r="H12" s="35"/>
+      <c r="I12" s="31" t="s">
+        <v>309</v>
+      </c>
+      <c r="J12" s="35"/>
+      <c r="K12" s="35"/>
+      <c r="L12" s="35"/>
+      <c r="M12" s="35"/>
+      <c r="N12" s="35"/>
+      <c r="O12" s="35"/>
+      <c r="P12" s="35"/>
+      <c r="Q12" s="35"/>
+    </row>
+    <row r="13" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="34" t="s">
         <v>259</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-    </row>
-    <row r="9" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-    </row>
-    <row r="10" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-    </row>
-    <row r="11" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-    </row>
-    <row r="12" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-    </row>
-    <row r="13" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-    </row>
-    <row r="14" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-    </row>
-    <row r="15" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-    </row>
-    <row r="16" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-    </row>
-    <row r="17" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-    </row>
-    <row r="18" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-    </row>
-    <row r="19" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-    </row>
-    <row r="20" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-    </row>
-    <row r="22" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="9"/>
-    </row>
-    <row r="23" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-    </row>
-    <row r="24" spans="2:15" s="5" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="23"/>
-      <c r="C24" s="23"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="23"/>
-      <c r="F24" s="23"/>
-      <c r="G24" s="23"/>
-      <c r="H24" s="23"/>
-      <c r="I24" s="23"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-    </row>
-    <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="29"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="27"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="27"/>
-      <c r="J25" s="9"/>
-    </row>
-    <row r="26" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B26" s="67"/>
-      <c r="C26" s="27"/>
-      <c r="D26" s="27"/>
-      <c r="E26" s="27"/>
-      <c r="F26" s="27"/>
-      <c r="G26" s="27"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="9"/>
-    </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B27" s="22"/>
-      <c r="C27" s="27"/>
-      <c r="D27" s="27"/>
-      <c r="E27" s="27"/>
-      <c r="F27" s="27"/>
-      <c r="G27" s="27"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="27"/>
-    </row>
-    <row r="28" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B28" s="68"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="27"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="27"/>
-    </row>
-    <row r="29" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B29" s="27"/>
-      <c r="C29" s="27"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
-      <c r="F29" s="27"/>
-      <c r="G29" s="27"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="27"/>
-    </row>
-    <row r="30" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B30" s="27"/>
-      <c r="C30" s="27"/>
-      <c r="D30" s="27"/>
-      <c r="E30" s="27"/>
-      <c r="F30" s="27"/>
-      <c r="G30" s="27"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="27"/>
-    </row>
-    <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="29"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="27"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="27"/>
-    </row>
-    <row r="32" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B32" s="27"/>
-      <c r="C32" s="27"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-    </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B33" s="27"/>
-      <c r="C33" s="27"/>
-      <c r="D33" s="27"/>
-      <c r="E33" s="27"/>
-      <c r="F33" s="27"/>
-      <c r="G33" s="27"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="27"/>
-    </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="29"/>
-      <c r="I34" s="27"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B35" s="27"/>
-      <c r="C35" s="27"/>
-      <c r="D35" s="27"/>
-      <c r="E35" s="27"/>
-      <c r="F35" s="27"/>
-      <c r="G35" s="27"/>
-      <c r="H35" s="29"/>
-      <c r="I35" s="27"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B36" s="27"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="27"/>
-      <c r="E36" s="27"/>
-      <c r="F36" s="27"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="29"/>
-      <c r="I36" s="27"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="27"/>
-      <c r="H37" s="27"/>
-      <c r="I37" s="27"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B38" s="27"/>
-      <c r="C38" s="27"/>
-      <c r="D38" s="27"/>
-      <c r="E38" s="27"/>
-      <c r="F38" s="27"/>
-      <c r="G38" s="27"/>
-      <c r="H38" s="27"/>
-      <c r="I38" s="27"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B39" s="27"/>
-      <c r="C39" s="27"/>
-      <c r="D39" s="27"/>
-      <c r="E39" s="27"/>
-      <c r="F39" s="27"/>
-      <c r="G39" s="27"/>
-      <c r="H39" s="29"/>
-      <c r="I39" s="27"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="27"/>
-      <c r="H40" s="29"/>
-      <c r="I40" s="27"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
-      <c r="D41" s="27"/>
-      <c r="E41" s="27"/>
-      <c r="F41" s="27"/>
-      <c r="G41" s="27"/>
-      <c r="H41" s="29"/>
-      <c r="I41" s="27"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B42" s="27"/>
-      <c r="C42" s="27"/>
-      <c r="D42" s="27"/>
-      <c r="E42" s="27"/>
-      <c r="F42" s="27"/>
-      <c r="G42" s="27"/>
-      <c r="H42" s="27"/>
-      <c r="I42" s="27"/>
-    </row>
-    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B43" s="27"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="27"/>
-      <c r="E43" s="27"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="27"/>
-      <c r="H43" s="27"/>
-      <c r="I43" s="27"/>
-    </row>
-    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B44" s="22"/>
-      <c r="C44" s="27"/>
-      <c r="D44" s="27"/>
-      <c r="E44" s="27"/>
-      <c r="F44" s="27"/>
-      <c r="G44" s="27"/>
-      <c r="H44" s="27"/>
-      <c r="I44" s="27"/>
-    </row>
-    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B45" s="27"/>
-      <c r="C45" s="25"/>
-      <c r="D45" s="27"/>
-      <c r="E45" s="27"/>
-      <c r="F45" s="27"/>
-      <c r="G45" s="27"/>
-      <c r="H45" s="27"/>
-      <c r="I45" s="27"/>
-    </row>
-    <row r="46" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B46" s="27"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="27"/>
-      <c r="E46" s="27"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="27"/>
-      <c r="H46" s="27"/>
-      <c r="I46" s="27"/>
-    </row>
-    <row r="47" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B47" s="27"/>
+      <c r="C13" s="35"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
+      <c r="G13" s="34" t="s">
+        <v>335</v>
+      </c>
+      <c r="H13" s="66"/>
+      <c r="I13" s="35" t="s">
+        <v>306</v>
+      </c>
+      <c r="J13" s="35"/>
+      <c r="K13" s="35"/>
+      <c r="L13" s="35"/>
+      <c r="M13" s="35"/>
+      <c r="N13" s="35"/>
+      <c r="O13" s="35"/>
+      <c r="P13" s="35"/>
+      <c r="Q13" s="35"/>
+    </row>
+    <row r="14" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="34" t="s">
+        <v>316</v>
+      </c>
+      <c r="H14" s="35"/>
+      <c r="I14" s="35" t="s">
+        <v>307</v>
+      </c>
+      <c r="J14" s="35"/>
+      <c r="K14" s="35"/>
+      <c r="L14" s="35"/>
+      <c r="M14" s="35"/>
+      <c r="N14" s="35"/>
+      <c r="O14" s="35"/>
+      <c r="P14" s="35"/>
+      <c r="Q14" s="35"/>
+    </row>
+    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="35"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="67"/>
+      <c r="H15" s="68"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="35"/>
+      <c r="L15" s="35"/>
+      <c r="M15" s="35"/>
+      <c r="N15" s="35"/>
+      <c r="O15" s="35"/>
+      <c r="P15" s="35"/>
+      <c r="Q15" s="35"/>
+    </row>
+    <row r="16" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="35"/>
+      <c r="C16" s="35"/>
+      <c r="D16" s="35"/>
+      <c r="E16" s="35"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="35"/>
+      <c r="O16" s="35"/>
+      <c r="P16" s="35"/>
+      <c r="Q16" s="35"/>
+    </row>
+    <row r="17" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="35"/>
+      <c r="C17" s="35"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="35"/>
+      <c r="J17" s="35"/>
+      <c r="K17" s="35"/>
+      <c r="L17" s="35"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="35"/>
+      <c r="O17" s="35"/>
+      <c r="P17" s="35"/>
+      <c r="Q17" s="35"/>
+    </row>
+    <row r="18" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="35"/>
+      <c r="C18" s="35"/>
+      <c r="D18" s="35"/>
+      <c r="E18" s="35"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
+      <c r="N18" s="35"/>
+      <c r="O18" s="35"/>
+      <c r="P18" s="35"/>
+      <c r="Q18" s="35"/>
+    </row>
+    <row r="19" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="35"/>
+      <c r="I19" s="35"/>
+      <c r="J19" s="35"/>
+      <c r="K19" s="35"/>
+      <c r="L19" s="35"/>
+      <c r="M19" s="35"/>
+      <c r="N19" s="35"/>
+      <c r="O19" s="35"/>
+      <c r="P19" s="35"/>
+      <c r="Q19" s="35"/>
+    </row>
+    <row r="20" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="35"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="35"/>
+    </row>
+    <row r="21" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B21" s="35"/>
+      <c r="C21" s="35"/>
+      <c r="D21" s="35"/>
+      <c r="E21" s="35"/>
+      <c r="F21" s="35"/>
+      <c r="G21" s="35"/>
+      <c r="H21" s="35"/>
+      <c r="I21" s="35"/>
+      <c r="J21" s="35"/>
+      <c r="K21" s="35"/>
+      <c r="L21" s="35"/>
+      <c r="M21" s="35"/>
+      <c r="N21" s="35"/>
+      <c r="O21" s="35"/>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="35"/>
+    </row>
+    <row r="22" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="35"/>
+      <c r="C22" s="35"/>
+      <c r="D22" s="35"/>
+      <c r="E22" s="35"/>
+      <c r="F22" s="35"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
+      <c r="K22" s="35"/>
+      <c r="L22" s="35"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="35"/>
+      <c r="O22" s="35"/>
+      <c r="P22" s="35"/>
+      <c r="Q22" s="35"/>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B24" s="22"/>
+      <c r="C24" s="22"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="28"/>
+      <c r="I24" s="28"/>
+      <c r="J24" s="28"/>
+      <c r="K24" s="31"/>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A25" s="31"/>
+      <c r="B25" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="G25" s="27" t="s">
+        <v>290</v>
+      </c>
+      <c r="K25" s="31"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+    </row>
+    <row r="26" spans="1:17" s="23" customFormat="1" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="31"/>
+      <c r="B26" s="57" t="s">
+        <v>283</v>
+      </c>
+      <c r="G26" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B27" s="57" t="s">
+        <v>284</v>
+      </c>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="K27" s="31"/>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B28" s="58"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="G28" s="27" t="s">
+        <v>292</v>
+      </c>
+      <c r="K28" s="31"/>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B29" s="22"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="G29" s="27" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B30" s="59" t="s">
+        <v>344</v>
+      </c>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="G30" s="29" t="s">
+        <v>294</v>
+      </c>
+      <c r="H30" s="29"/>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B31" s="23" t="s">
+        <v>345</v>
+      </c>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="B32" s="23" t="s">
+        <v>346</v>
+      </c>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+    </row>
+    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B33" s="57"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+    </row>
+    <row r="34" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="G34" s="24"/>
+      <c r="H34" s="24"/>
+      <c r="I34" s="24"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="24"/>
+      <c r="L34" s="24"/>
+      <c r="M34" s="24"/>
+      <c r="N34" s="24"/>
+    </row>
+    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I36" s="29"/>
+    </row>
+    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I37" s="29"/>
+    </row>
+    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I38" s="29"/>
+    </row>
+    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I41" s="29"/>
+    </row>
+    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I42" s="29"/>
+    </row>
+    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="I43" s="29"/>
+    </row>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B46" s="22"/>
+    </row>
+    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C47" s="25"/>
-      <c r="D47" s="27"/>
-      <c r="E47" s="27"/>
-      <c r="F47" s="27"/>
-      <c r="G47" s="27"/>
-      <c r="H47" s="27"/>
-      <c r="I47" s="27"/>
-    </row>
-    <row r="48" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B48" s="27"/>
+    </row>
+    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
       <c r="C48" s="25"/>
-      <c r="D48" s="27"/>
-      <c r="E48" s="27"/>
-      <c r="F48" s="27"/>
-      <c r="G48" s="27"/>
-      <c r="H48" s="27"/>
-      <c r="I48" s="27"/>
-    </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B49" s="27"/>
-      <c r="C49" s="27"/>
-      <c r="D49" s="27"/>
-      <c r="E49" s="27"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="27"/>
-      <c r="H49" s="27"/>
-      <c r="I49" s="27"/>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B50" s="27"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="27"/>
-      <c r="E50" s="27"/>
-      <c r="F50" s="27"/>
-      <c r="G50" s="27"/>
-      <c r="H50" s="27"/>
-      <c r="I50" s="27"/>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="27"/>
-      <c r="B51" s="27"/>
-      <c r="C51" s="27"/>
-      <c r="D51" s="27"/>
-      <c r="E51" s="27"/>
-      <c r="F51" s="27"/>
-      <c r="G51" s="27"/>
-      <c r="H51" s="27"/>
-      <c r="I51" s="27"/>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" s="27"/>
-      <c r="B52" s="27"/>
-      <c r="C52" s="27"/>
-      <c r="D52" s="27"/>
-      <c r="E52" s="27"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="27"/>
-      <c r="H52" s="27"/>
-      <c r="I52" s="27"/>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A53" s="27"/>
-      <c r="B53" s="27"/>
-      <c r="C53" s="27"/>
-      <c r="D53" s="27"/>
-      <c r="E53" s="27"/>
-      <c r="F53" s="27"/>
-      <c r="G53" s="27"/>
-      <c r="H53" s="29"/>
-      <c r="I53" s="27"/>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" s="52"/>
-      <c r="B54" s="52"/>
-      <c r="C54" s="52"/>
-      <c r="D54" s="52"/>
-      <c r="E54" s="52"/>
-      <c r="F54" s="52"/>
-      <c r="G54" s="52"/>
-      <c r="H54" s="53"/>
-      <c r="I54" s="52"/>
-      <c r="J54" s="54"/>
-      <c r="K54" s="54"/>
-      <c r="L54" s="54"/>
-      <c r="M54" s="54"/>
-      <c r="N54" s="54"/>
-      <c r="O54" s="54"/>
-      <c r="P54" s="54"/>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="52"/>
-      <c r="B55" s="52"/>
-      <c r="C55" s="52"/>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="52"/>
-      <c r="H55" s="53"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="54"/>
-      <c r="K55" s="54"/>
-      <c r="L55" s="54"/>
-      <c r="M55" s="54"/>
-      <c r="N55" s="54"/>
-      <c r="O55" s="54"/>
-      <c r="P55" s="54"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="55"/>
-      <c r="B56" s="53"/>
-      <c r="C56" s="52"/>
-      <c r="D56" s="52"/>
-      <c r="E56" s="52"/>
-      <c r="F56" s="52"/>
-      <c r="G56" s="52"/>
-      <c r="H56" s="52"/>
-      <c r="I56" s="52"/>
-      <c r="J56" s="54"/>
-      <c r="K56" s="54"/>
-      <c r="L56" s="54"/>
-      <c r="M56" s="54"/>
-      <c r="N56" s="54"/>
-      <c r="O56" s="54"/>
-      <c r="P56" s="54"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A57" s="55"/>
-      <c r="B57" s="53"/>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="52"/>
-      <c r="H57" s="52"/>
-      <c r="I57" s="52"/>
-      <c r="J57" s="54"/>
-      <c r="K57" s="54"/>
-      <c r="L57" s="54"/>
-      <c r="M57" s="54"/>
-      <c r="N57" s="54"/>
-      <c r="O57" s="54"/>
-      <c r="P57" s="54"/>
-    </row>
-    <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="55"/>
-      <c r="B58" s="52"/>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-      <c r="J58" s="54"/>
-      <c r="K58" s="54"/>
-      <c r="L58" s="54"/>
-      <c r="M58" s="54"/>
-      <c r="N58" s="54"/>
-      <c r="O58" s="54"/>
-      <c r="P58" s="54"/>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A59" s="55"/>
-      <c r="B59" s="53"/>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-      <c r="J59" s="54"/>
-      <c r="K59" s="54"/>
-      <c r="L59" s="54"/>
-      <c r="M59" s="54"/>
-      <c r="N59" s="54"/>
-      <c r="O59" s="54"/>
-      <c r="P59" s="54"/>
-    </row>
-    <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="55"/>
-      <c r="B60" s="53"/>
-      <c r="C60" s="54"/>
-      <c r="D60" s="54"/>
-      <c r="E60" s="54"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="52"/>
-      <c r="H60" s="52"/>
-      <c r="I60" s="52"/>
-      <c r="J60" s="54"/>
-      <c r="K60" s="54"/>
-      <c r="L60" s="54"/>
-      <c r="M60" s="54"/>
-      <c r="N60" s="54"/>
-      <c r="O60" s="54"/>
-      <c r="P60" s="54"/>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="55"/>
-      <c r="B61" s="53"/>
-      <c r="C61" s="54"/>
-      <c r="D61" s="54"/>
-      <c r="E61" s="54"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="52"/>
-      <c r="H61" s="52"/>
-      <c r="I61" s="52"/>
-      <c r="J61" s="54"/>
-      <c r="K61" s="54"/>
-      <c r="L61" s="54"/>
-      <c r="M61" s="54"/>
-      <c r="N61" s="54"/>
-      <c r="O61" s="54"/>
-      <c r="P61" s="54"/>
-    </row>
-    <row r="62" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A62" s="52"/>
-      <c r="B62" s="56"/>
-      <c r="C62" s="56"/>
-      <c r="D62" s="56"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="54"/>
-      <c r="H62" s="56"/>
-      <c r="I62" s="56"/>
-      <c r="J62" s="56"/>
-      <c r="K62" s="54"/>
-      <c r="L62" s="56"/>
-      <c r="M62" s="54"/>
-      <c r="N62" s="54"/>
-      <c r="O62" s="54"/>
-      <c r="P62" s="54"/>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A63" s="52"/>
-      <c r="B63" s="57"/>
-      <c r="C63" s="56"/>
-      <c r="D63" s="56"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="54"/>
-      <c r="H63" s="57"/>
-      <c r="I63" s="56"/>
-      <c r="J63" s="56"/>
-      <c r="K63" s="54"/>
-      <c r="L63" s="58"/>
-      <c r="M63" s="58"/>
-      <c r="N63" s="54"/>
-      <c r="O63" s="54"/>
-      <c r="P63" s="54"/>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A64" s="52"/>
-      <c r="B64" s="56"/>
-      <c r="C64" s="56"/>
-      <c r="D64" s="56"/>
-      <c r="E64" s="52"/>
-      <c r="F64" s="52"/>
-      <c r="G64" s="54"/>
-      <c r="H64" s="56"/>
-      <c r="I64" s="56"/>
-      <c r="J64" s="56"/>
-      <c r="K64" s="54"/>
-      <c r="L64" s="56"/>
-      <c r="M64" s="56"/>
-      <c r="N64" s="54"/>
-      <c r="O64" s="54"/>
-      <c r="P64" s="54"/>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A65" s="52"/>
-      <c r="B65" s="56"/>
-      <c r="C65" s="56"/>
-      <c r="D65" s="56"/>
-      <c r="E65" s="52"/>
-      <c r="F65" s="52"/>
-      <c r="G65" s="54"/>
-      <c r="H65" s="56"/>
-      <c r="I65" s="56"/>
-      <c r="J65" s="56"/>
-      <c r="K65" s="54"/>
-      <c r="L65" s="56"/>
-      <c r="M65" s="56"/>
-      <c r="N65" s="54"/>
-      <c r="O65" s="54"/>
-      <c r="P65" s="54"/>
-    </row>
-    <row r="66" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" s="52"/>
-      <c r="B66" s="56"/>
-      <c r="C66" s="56"/>
-      <c r="D66" s="56"/>
-      <c r="E66" s="52"/>
-      <c r="F66" s="52"/>
-      <c r="G66" s="54"/>
-      <c r="H66" s="56"/>
-      <c r="I66" s="56"/>
-      <c r="J66" s="56"/>
-      <c r="K66" s="54"/>
-      <c r="L66" s="56"/>
-      <c r="M66" s="56"/>
-      <c r="N66" s="54"/>
-      <c r="O66" s="54"/>
-      <c r="P66" s="54"/>
-    </row>
-    <row r="67" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A67" s="52"/>
-      <c r="B67" s="56"/>
-      <c r="C67" s="56"/>
-      <c r="D67" s="56"/>
-      <c r="E67" s="52"/>
-      <c r="F67" s="52"/>
-      <c r="G67" s="54"/>
-      <c r="H67" s="56"/>
-      <c r="I67" s="56"/>
-      <c r="J67" s="56"/>
-      <c r="K67" s="54"/>
-      <c r="L67" s="56"/>
-      <c r="M67" s="56"/>
-      <c r="N67" s="54"/>
-      <c r="O67" s="54"/>
-      <c r="P67" s="54"/>
-    </row>
-    <row r="68" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A68" s="52"/>
-      <c r="B68" s="52"/>
-      <c r="C68" s="52"/>
-      <c r="D68" s="52"/>
-      <c r="E68" s="52"/>
-      <c r="F68" s="52"/>
-      <c r="G68" s="54"/>
-      <c r="H68" s="52"/>
-      <c r="I68" s="52"/>
-      <c r="J68" s="52"/>
-      <c r="K68" s="54"/>
-      <c r="L68" s="56"/>
-      <c r="M68" s="56"/>
-      <c r="N68" s="54"/>
-      <c r="O68" s="54"/>
-      <c r="P68" s="54"/>
-    </row>
-    <row r="69" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A69" s="52"/>
-      <c r="B69" s="52"/>
-      <c r="C69" s="52"/>
-      <c r="D69" s="52"/>
-      <c r="E69" s="52"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="54"/>
-      <c r="H69" s="52"/>
-      <c r="I69" s="52"/>
-      <c r="J69" s="52"/>
-      <c r="K69" s="54"/>
-      <c r="L69" s="54"/>
-      <c r="M69" s="54"/>
-      <c r="N69" s="54"/>
-      <c r="O69" s="54"/>
-      <c r="P69" s="54"/>
-    </row>
-    <row r="70" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A70" s="52"/>
-      <c r="B70" s="56"/>
-      <c r="C70" s="56"/>
-      <c r="D70" s="56"/>
-      <c r="E70" s="54"/>
-      <c r="F70" s="56"/>
-      <c r="G70" s="54"/>
-      <c r="H70" s="56"/>
-      <c r="I70" s="56"/>
-      <c r="J70" s="56"/>
-      <c r="K70" s="54"/>
-      <c r="L70" s="54"/>
-      <c r="M70" s="54"/>
-      <c r="N70" s="54"/>
-      <c r="O70" s="54"/>
-      <c r="P70" s="54"/>
-    </row>
-    <row r="71" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A71" s="52"/>
-      <c r="B71" s="57"/>
-      <c r="C71" s="56"/>
-      <c r="D71" s="56"/>
-      <c r="E71" s="56"/>
-      <c r="F71" s="58"/>
-      <c r="G71" s="54"/>
-      <c r="H71" s="57"/>
-      <c r="I71" s="56"/>
-      <c r="J71" s="56"/>
-      <c r="K71" s="54"/>
-      <c r="L71" s="54"/>
-      <c r="M71" s="54"/>
-      <c r="N71" s="54"/>
-      <c r="O71" s="54"/>
-      <c r="P71" s="54"/>
-    </row>
-    <row r="72" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A72" s="52"/>
-      <c r="B72" s="56"/>
-      <c r="C72" s="56"/>
-      <c r="D72" s="56"/>
-      <c r="E72" s="59"/>
-      <c r="F72" s="56"/>
-      <c r="G72" s="54"/>
-      <c r="H72" s="56"/>
-      <c r="I72" s="56"/>
-      <c r="J72" s="56"/>
-      <c r="K72" s="54"/>
-      <c r="L72" s="54"/>
-      <c r="M72" s="54"/>
-      <c r="N72" s="54"/>
-      <c r="O72" s="54"/>
-      <c r="P72" s="54"/>
-    </row>
-    <row r="73" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A73" s="52"/>
-      <c r="B73" s="56"/>
-      <c r="C73" s="56"/>
-      <c r="D73" s="56"/>
-      <c r="E73" s="59"/>
-      <c r="F73" s="56"/>
-      <c r="G73" s="54"/>
-      <c r="H73" s="56"/>
-      <c r="I73" s="56"/>
-      <c r="J73" s="56"/>
-      <c r="K73" s="54"/>
-      <c r="L73" s="54"/>
-      <c r="M73" s="54"/>
-      <c r="N73" s="54"/>
-      <c r="O73" s="54"/>
-      <c r="P73" s="54"/>
-    </row>
-    <row r="74" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A74" s="52"/>
-      <c r="B74" s="56"/>
-      <c r="C74" s="56"/>
-      <c r="D74" s="56"/>
-      <c r="E74" s="59"/>
-      <c r="F74" s="56"/>
-      <c r="G74" s="54"/>
-      <c r="H74" s="56"/>
-      <c r="I74" s="56"/>
-      <c r="J74" s="56"/>
-      <c r="K74" s="54"/>
-      <c r="L74" s="54"/>
-      <c r="M74" s="54"/>
-      <c r="N74" s="54"/>
-      <c r="O74" s="54"/>
-      <c r="P74" s="54"/>
-    </row>
-    <row r="75" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A75" s="54"/>
-      <c r="B75" s="56"/>
-      <c r="C75" s="56"/>
-      <c r="D75" s="56"/>
-      <c r="E75" s="59"/>
-      <c r="F75" s="56"/>
-      <c r="G75" s="54"/>
-      <c r="H75" s="56"/>
-      <c r="I75" s="56"/>
-      <c r="J75" s="56"/>
-      <c r="K75" s="54"/>
-      <c r="L75" s="54"/>
-      <c r="M75" s="54"/>
-      <c r="N75" s="54"/>
-      <c r="O75" s="54"/>
-      <c r="P75" s="54"/>
-    </row>
-    <row r="76" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A76" s="54"/>
-      <c r="B76" s="56"/>
-      <c r="C76" s="56"/>
-      <c r="D76" s="56"/>
-      <c r="E76" s="59"/>
-      <c r="F76" s="56"/>
-      <c r="G76" s="54"/>
-      <c r="H76" s="54"/>
-      <c r="I76" s="52"/>
-      <c r="J76" s="54"/>
-      <c r="K76" s="54"/>
-      <c r="L76" s="54"/>
-      <c r="M76" s="54"/>
-      <c r="N76" s="54"/>
-      <c r="O76" s="54"/>
-      <c r="P76" s="54"/>
-    </row>
-    <row r="77" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A77" s="54"/>
-      <c r="B77" s="52"/>
-      <c r="C77" s="52"/>
-      <c r="D77" s="52"/>
-      <c r="E77" s="52"/>
-      <c r="F77" s="54"/>
-      <c r="G77" s="54"/>
-      <c r="H77" s="54"/>
-      <c r="I77" s="52"/>
-      <c r="J77" s="54"/>
-      <c r="K77" s="54"/>
-      <c r="L77" s="54"/>
-      <c r="M77" s="54"/>
-      <c r="N77" s="54"/>
-      <c r="O77" s="54"/>
-      <c r="P77" s="54"/>
-    </row>
-    <row r="78" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A78" s="54"/>
-      <c r="B78" s="52"/>
-      <c r="C78" s="52"/>
-      <c r="D78" s="52"/>
-      <c r="E78" s="52"/>
-      <c r="F78" s="54"/>
-      <c r="G78" s="54"/>
-      <c r="H78" s="54"/>
-      <c r="I78" s="52"/>
-      <c r="J78" s="54"/>
-      <c r="K78" s="54"/>
-      <c r="L78" s="54"/>
-      <c r="M78" s="54"/>
-      <c r="N78" s="54"/>
-      <c r="O78" s="54"/>
-      <c r="P78" s="54"/>
-    </row>
-    <row r="79" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A79" s="52"/>
-      <c r="B79" s="56"/>
-      <c r="C79" s="60"/>
-      <c r="D79" s="60"/>
-      <c r="E79" s="52"/>
-      <c r="F79" s="52"/>
-      <c r="G79" s="52"/>
-      <c r="H79" s="52"/>
-      <c r="I79" s="52"/>
-      <c r="J79" s="54"/>
-      <c r="K79" s="54"/>
-      <c r="L79" s="54"/>
-      <c r="M79" s="54"/>
-      <c r="N79" s="54"/>
-      <c r="O79" s="54"/>
-      <c r="P79" s="54"/>
-    </row>
-    <row r="80" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A80" s="52"/>
-      <c r="B80" s="57"/>
-      <c r="C80" s="56"/>
-      <c r="D80" s="56"/>
-      <c r="E80" s="56"/>
-      <c r="F80" s="61"/>
-      <c r="G80" s="52"/>
-      <c r="H80" s="56"/>
-      <c r="I80" s="56"/>
-      <c r="J80" s="56"/>
-      <c r="K80" s="54"/>
-      <c r="L80" s="54"/>
-      <c r="M80" s="54"/>
-      <c r="N80" s="54"/>
-      <c r="O80" s="54"/>
-      <c r="P80" s="54"/>
-    </row>
-    <row r="81" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A81" s="52"/>
-      <c r="B81" s="56"/>
-      <c r="C81" s="56"/>
-      <c r="D81" s="56"/>
-      <c r="E81" s="56"/>
-      <c r="F81" s="56"/>
-      <c r="G81" s="52"/>
-      <c r="H81" s="57"/>
-      <c r="I81" s="56"/>
-      <c r="J81" s="58"/>
-      <c r="K81" s="54"/>
-      <c r="L81" s="54"/>
-      <c r="M81" s="54"/>
-      <c r="N81" s="54"/>
-      <c r="O81" s="54"/>
-      <c r="P81" s="54"/>
-    </row>
-    <row r="82" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A82" s="52"/>
-      <c r="B82" s="56"/>
-      <c r="C82" s="56"/>
-      <c r="D82" s="56"/>
-      <c r="E82" s="56"/>
-      <c r="F82" s="56"/>
-      <c r="G82" s="52"/>
-      <c r="H82" s="56"/>
-      <c r="I82" s="56"/>
-      <c r="J82" s="56"/>
-      <c r="K82" s="54"/>
-      <c r="L82" s="54"/>
-      <c r="M82" s="54"/>
-      <c r="N82" s="54"/>
-      <c r="O82" s="54"/>
-      <c r="P82" s="54"/>
-    </row>
-    <row r="83" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A83" s="52"/>
-      <c r="B83" s="56"/>
-      <c r="C83" s="56"/>
-      <c r="D83" s="56"/>
-      <c r="E83" s="56"/>
-      <c r="F83" s="56"/>
-      <c r="G83" s="52"/>
-      <c r="H83" s="56"/>
-      <c r="I83" s="56"/>
-      <c r="J83" s="56"/>
-      <c r="K83" s="54"/>
-      <c r="L83" s="54"/>
-      <c r="M83" s="54"/>
-      <c r="N83" s="54"/>
-      <c r="O83" s="54"/>
-      <c r="P83" s="54"/>
-    </row>
-    <row r="84" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A84" s="52"/>
-      <c r="B84" s="56"/>
-      <c r="C84" s="56"/>
-      <c r="D84" s="56"/>
-      <c r="E84" s="56"/>
-      <c r="F84" s="56"/>
-      <c r="G84" s="52"/>
-      <c r="H84" s="56"/>
-      <c r="I84" s="56"/>
-      <c r="J84" s="56"/>
-      <c r="K84" s="54"/>
-      <c r="L84" s="54"/>
-      <c r="M84" s="54"/>
-      <c r="N84" s="54"/>
-      <c r="O84" s="54"/>
-      <c r="P84" s="54"/>
-    </row>
-    <row r="85" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A85" s="52"/>
-      <c r="B85" s="56"/>
-      <c r="C85" s="56"/>
-      <c r="D85" s="56"/>
-      <c r="E85" s="56"/>
-      <c r="F85" s="56"/>
-      <c r="G85" s="52"/>
-      <c r="H85" s="56"/>
-      <c r="I85" s="56"/>
-      <c r="J85" s="56"/>
-      <c r="K85" s="54"/>
-      <c r="L85" s="54"/>
-      <c r="M85" s="54"/>
-      <c r="N85" s="54"/>
-      <c r="O85" s="54"/>
-      <c r="P85" s="54"/>
-    </row>
-    <row r="86" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A86" s="52"/>
-      <c r="B86" s="56"/>
-      <c r="C86" s="56"/>
-      <c r="D86" s="56"/>
-      <c r="E86" s="56"/>
-      <c r="F86" s="56"/>
-      <c r="G86" s="52"/>
-      <c r="H86" s="56"/>
-      <c r="I86" s="56"/>
-      <c r="J86" s="56"/>
-      <c r="K86" s="54"/>
-      <c r="L86" s="54"/>
-      <c r="M86" s="54"/>
-      <c r="N86" s="54"/>
-      <c r="O86" s="54"/>
-      <c r="P86" s="54"/>
-    </row>
-    <row r="87" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A87" s="52"/>
-      <c r="B87" s="52"/>
-      <c r="C87" s="52"/>
-      <c r="D87" s="52"/>
-      <c r="E87" s="52"/>
-      <c r="F87" s="52"/>
-      <c r="G87" s="52"/>
-      <c r="H87" s="56"/>
-      <c r="I87" s="56"/>
-      <c r="J87" s="56"/>
-      <c r="K87" s="54"/>
-      <c r="L87" s="54"/>
-      <c r="M87" s="54"/>
-      <c r="N87" s="54"/>
-      <c r="O87" s="54"/>
-      <c r="P87" s="54"/>
-    </row>
-    <row r="88" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A88" s="52"/>
-      <c r="B88" s="52"/>
-      <c r="C88" s="52"/>
-      <c r="D88" s="52"/>
-      <c r="E88" s="52"/>
-      <c r="F88" s="52"/>
-      <c r="G88" s="52"/>
-      <c r="H88" s="56"/>
-      <c r="I88" s="56"/>
-      <c r="J88" s="56"/>
-      <c r="K88" s="54"/>
-      <c r="L88" s="54"/>
-      <c r="M88" s="54"/>
-      <c r="N88" s="54"/>
-      <c r="O88" s="54"/>
-      <c r="P88" s="54"/>
-    </row>
-    <row r="89" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A89" s="52"/>
-      <c r="B89" s="56"/>
-      <c r="C89" s="56"/>
-      <c r="D89" s="52"/>
-      <c r="E89" s="52"/>
-      <c r="F89" s="52"/>
-      <c r="G89" s="52"/>
-      <c r="H89" s="56"/>
-      <c r="I89" s="56"/>
-      <c r="J89" s="56"/>
-      <c r="K89" s="54"/>
-      <c r="L89" s="54"/>
-      <c r="M89" s="54"/>
-      <c r="N89" s="54"/>
-      <c r="O89" s="54"/>
-      <c r="P89" s="54"/>
-    </row>
-    <row r="90" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A90" s="54"/>
-      <c r="B90" s="57"/>
-      <c r="C90" s="58"/>
-      <c r="D90" s="61"/>
-      <c r="E90" s="54"/>
-      <c r="F90" s="52"/>
-      <c r="G90" s="52"/>
-      <c r="H90" s="52"/>
-      <c r="I90" s="52"/>
-      <c r="J90" s="54"/>
-      <c r="K90" s="54"/>
-      <c r="L90" s="54"/>
-      <c r="M90" s="54"/>
-      <c r="N90" s="54"/>
-      <c r="O90" s="54"/>
-      <c r="P90" s="54"/>
-    </row>
-    <row r="91" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A91" s="54"/>
-      <c r="B91" s="56"/>
-      <c r="C91" s="56"/>
-      <c r="D91" s="56"/>
-      <c r="E91" s="54"/>
-      <c r="F91" s="52"/>
-      <c r="G91" s="52"/>
-      <c r="H91" s="52"/>
-      <c r="I91" s="52"/>
-      <c r="J91" s="54"/>
-      <c r="K91" s="54"/>
-      <c r="L91" s="54"/>
-      <c r="M91" s="54"/>
-      <c r="N91" s="54"/>
-      <c r="O91" s="54"/>
-      <c r="P91" s="54"/>
-    </row>
-    <row r="92" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A92" s="54"/>
-      <c r="B92" s="56"/>
-      <c r="C92" s="56"/>
-      <c r="D92" s="56"/>
-      <c r="E92" s="54"/>
-      <c r="F92" s="52"/>
-      <c r="G92" s="52"/>
-      <c r="H92" s="52"/>
-      <c r="I92" s="52"/>
-      <c r="J92" s="54"/>
-      <c r="K92" s="54"/>
-      <c r="L92" s="54"/>
-      <c r="M92" s="54"/>
-      <c r="N92" s="54"/>
-      <c r="O92" s="54"/>
-      <c r="P92" s="54"/>
-    </row>
-    <row r="93" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A93" s="54"/>
-      <c r="B93" s="56"/>
-      <c r="C93" s="56"/>
-      <c r="D93" s="56"/>
-      <c r="E93" s="54"/>
-      <c r="F93" s="52"/>
-      <c r="G93" s="52"/>
-      <c r="H93" s="52"/>
-      <c r="I93" s="52"/>
-      <c r="J93" s="54"/>
-      <c r="K93" s="54"/>
-      <c r="L93" s="54"/>
-      <c r="M93" s="54"/>
-      <c r="N93" s="54"/>
-      <c r="O93" s="54"/>
-      <c r="P93" s="54"/>
-    </row>
-    <row r="94" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A94" s="54"/>
-      <c r="B94" s="56"/>
-      <c r="C94" s="56"/>
-      <c r="D94" s="56"/>
-      <c r="E94" s="54"/>
-      <c r="F94" s="52"/>
-      <c r="G94" s="52"/>
-      <c r="H94" s="52"/>
-      <c r="I94" s="52"/>
-      <c r="J94" s="54"/>
-      <c r="K94" s="54"/>
-      <c r="L94" s="54"/>
-      <c r="M94" s="54"/>
-      <c r="N94" s="54"/>
-      <c r="O94" s="54"/>
-      <c r="P94" s="54"/>
-    </row>
-    <row r="95" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A95" s="54"/>
-      <c r="B95" s="56"/>
-      <c r="C95" s="56"/>
-      <c r="D95" s="56"/>
-      <c r="E95" s="54"/>
-      <c r="F95" s="52"/>
-      <c r="G95" s="52"/>
-      <c r="H95" s="52"/>
-      <c r="I95" s="52"/>
-      <c r="J95" s="54"/>
-      <c r="K95" s="54"/>
-      <c r="L95" s="54"/>
-      <c r="M95" s="54"/>
-      <c r="N95" s="54"/>
-      <c r="O95" s="54"/>
-      <c r="P95" s="54"/>
-    </row>
-    <row r="96" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A96" s="54"/>
-      <c r="B96" s="56"/>
-      <c r="C96" s="56"/>
-      <c r="D96" s="56"/>
-      <c r="E96" s="54"/>
-      <c r="F96" s="52"/>
-      <c r="G96" s="52"/>
-      <c r="H96" s="52"/>
-      <c r="I96" s="52"/>
-      <c r="J96" s="54"/>
-      <c r="K96" s="54"/>
-      <c r="L96" s="54"/>
-      <c r="M96" s="54"/>
-      <c r="N96" s="54"/>
-      <c r="O96" s="54"/>
-      <c r="P96" s="54"/>
-    </row>
-    <row r="97" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A97" s="54"/>
-      <c r="B97" s="52"/>
-      <c r="C97" s="52"/>
-      <c r="D97" s="52"/>
-      <c r="E97" s="52"/>
-      <c r="F97" s="52"/>
-      <c r="G97" s="52"/>
-      <c r="H97" s="52"/>
-      <c r="I97" s="52"/>
-      <c r="J97" s="54"/>
-      <c r="K97" s="54"/>
-      <c r="L97" s="54"/>
-      <c r="M97" s="54"/>
-      <c r="N97" s="54"/>
-      <c r="O97" s="54"/>
-      <c r="P97" s="54"/>
-    </row>
-    <row r="98" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A98" s="54"/>
-      <c r="B98" s="52"/>
-      <c r="C98" s="52"/>
-      <c r="D98" s="52"/>
-      <c r="E98" s="52"/>
-      <c r="F98" s="52"/>
-      <c r="G98" s="52"/>
-      <c r="H98" s="52"/>
-      <c r="I98" s="52"/>
-      <c r="J98" s="54"/>
-      <c r="K98" s="54"/>
-      <c r="L98" s="54"/>
-      <c r="M98" s="54"/>
-      <c r="N98" s="54"/>
-      <c r="O98" s="54"/>
-      <c r="P98" s="54"/>
-    </row>
-    <row r="99" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A99" s="54"/>
-      <c r="B99" s="52"/>
-      <c r="C99" s="52"/>
-      <c r="D99" s="52"/>
-      <c r="E99" s="52"/>
-      <c r="F99" s="52"/>
-      <c r="G99" s="52"/>
-      <c r="H99" s="52"/>
-      <c r="I99" s="52"/>
-      <c r="J99" s="54"/>
-      <c r="K99" s="54"/>
-      <c r="L99" s="54"/>
-      <c r="M99" s="54"/>
-      <c r="N99" s="54"/>
-      <c r="O99" s="54"/>
-      <c r="P99" s="54"/>
-    </row>
-    <row r="100" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A100" s="54"/>
-      <c r="B100" s="53"/>
-      <c r="C100" s="52"/>
-      <c r="D100" s="52"/>
-      <c r="E100" s="52"/>
-      <c r="F100" s="52"/>
-      <c r="G100" s="52"/>
-      <c r="H100" s="52"/>
-      <c r="I100" s="52"/>
-      <c r="J100" s="54"/>
-      <c r="K100" s="54"/>
-      <c r="L100" s="54"/>
-      <c r="M100" s="54"/>
-      <c r="N100" s="54"/>
-      <c r="O100" s="54"/>
-      <c r="P100" s="54"/>
-    </row>
-    <row r="101" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A101" s="54"/>
-      <c r="B101" s="53"/>
-      <c r="C101" s="52"/>
-      <c r="D101" s="52"/>
-      <c r="E101" s="52"/>
-      <c r="F101" s="52"/>
-      <c r="G101" s="52"/>
-      <c r="H101" s="52"/>
-      <c r="I101" s="52"/>
-      <c r="J101" s="54"/>
-      <c r="K101" s="54"/>
-      <c r="L101" s="54"/>
-      <c r="M101" s="54"/>
-      <c r="N101" s="54"/>
-      <c r="O101" s="54"/>
-      <c r="P101" s="54"/>
-    </row>
-    <row r="102" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A102" s="54"/>
-      <c r="B102" s="52"/>
-      <c r="C102" s="54"/>
-      <c r="D102" s="54"/>
-      <c r="E102" s="54"/>
-      <c r="F102" s="52"/>
-      <c r="G102" s="52"/>
-      <c r="H102" s="52"/>
-      <c r="I102" s="52"/>
-      <c r="J102" s="54"/>
-      <c r="K102" s="54"/>
-      <c r="L102" s="54"/>
-      <c r="M102" s="54"/>
-      <c r="N102" s="54"/>
-      <c r="O102" s="54"/>
-      <c r="P102" s="54"/>
-    </row>
-    <row r="103" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A103" s="54"/>
-      <c r="B103" s="62"/>
-      <c r="C103" s="54"/>
-      <c r="D103" s="54"/>
-      <c r="E103" s="54"/>
-      <c r="F103" s="52"/>
-      <c r="G103" s="52"/>
-      <c r="H103" s="52"/>
-      <c r="I103" s="52"/>
-      <c r="J103" s="54"/>
-      <c r="K103" s="54"/>
-      <c r="L103" s="54"/>
-      <c r="M103" s="54"/>
-      <c r="N103" s="54"/>
-      <c r="O103" s="54"/>
-      <c r="P103" s="54"/>
-    </row>
-    <row r="104" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A104" s="54"/>
-      <c r="B104" s="54"/>
-      <c r="C104" s="54"/>
-      <c r="D104" s="54"/>
-      <c r="E104" s="54"/>
-      <c r="F104" s="52"/>
-      <c r="G104" s="56"/>
-      <c r="H104" s="52"/>
-      <c r="I104" s="52"/>
-      <c r="J104" s="54"/>
-      <c r="K104" s="54"/>
-      <c r="L104" s="54"/>
-      <c r="M104" s="54"/>
-      <c r="N104" s="54"/>
-      <c r="O104" s="54"/>
-      <c r="P104" s="54"/>
-    </row>
-    <row r="105" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A105" s="54"/>
-      <c r="B105" s="56"/>
-      <c r="C105" s="52"/>
-      <c r="D105" s="52"/>
-      <c r="E105" s="52"/>
-      <c r="F105" s="52"/>
-      <c r="G105" s="59"/>
-      <c r="H105" s="59"/>
-      <c r="I105" s="52"/>
-      <c r="J105" s="54"/>
-      <c r="K105" s="54"/>
-      <c r="L105" s="54"/>
-      <c r="M105" s="54"/>
-      <c r="N105" s="54"/>
-      <c r="O105" s="54"/>
-      <c r="P105" s="54"/>
-    </row>
-    <row r="106" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A106" s="54"/>
-      <c r="B106" s="57"/>
-      <c r="C106" s="56"/>
-      <c r="D106" s="56"/>
-      <c r="E106" s="52"/>
-      <c r="F106" s="52"/>
-      <c r="G106" s="58"/>
-      <c r="H106" s="58"/>
-      <c r="I106" s="52"/>
-      <c r="J106" s="54"/>
-      <c r="K106" s="54"/>
-      <c r="L106" s="54"/>
-      <c r="M106" s="54"/>
-      <c r="N106" s="54"/>
-      <c r="O106" s="54"/>
-      <c r="P106" s="54"/>
-    </row>
-    <row r="107" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A107" s="54"/>
-      <c r="B107" s="56"/>
-      <c r="C107" s="56"/>
-      <c r="D107" s="56"/>
-      <c r="E107" s="52"/>
-      <c r="F107" s="52"/>
-      <c r="G107" s="56"/>
-      <c r="H107" s="56"/>
-      <c r="I107" s="52"/>
-      <c r="J107" s="54"/>
-      <c r="K107" s="54"/>
-      <c r="L107" s="54"/>
-      <c r="M107" s="54"/>
-      <c r="N107" s="54"/>
-      <c r="O107" s="54"/>
-      <c r="P107" s="54"/>
-    </row>
-    <row r="108" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A108" s="54"/>
-      <c r="B108" s="56"/>
-      <c r="C108" s="56"/>
-      <c r="D108" s="56"/>
-      <c r="E108" s="52"/>
-      <c r="F108" s="52"/>
-      <c r="G108" s="56"/>
-      <c r="H108" s="56"/>
-      <c r="I108" s="52"/>
-      <c r="J108" s="54"/>
-      <c r="K108" s="54"/>
-      <c r="L108" s="54"/>
-      <c r="M108" s="54"/>
-      <c r="N108" s="54"/>
-      <c r="O108" s="54"/>
-      <c r="P108" s="54"/>
-    </row>
-    <row r="109" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A109" s="54"/>
-      <c r="B109" s="56"/>
-      <c r="C109" s="56"/>
-      <c r="D109" s="56"/>
-      <c r="E109" s="52"/>
-      <c r="F109" s="52"/>
-      <c r="G109" s="56"/>
-      <c r="H109" s="56"/>
-      <c r="I109" s="52"/>
-      <c r="J109" s="54"/>
-      <c r="K109" s="54"/>
-      <c r="L109" s="54"/>
-      <c r="M109" s="54"/>
-      <c r="N109" s="54"/>
-      <c r="O109" s="54"/>
-      <c r="P109" s="54"/>
-    </row>
-    <row r="110" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A110" s="54"/>
-      <c r="B110" s="56"/>
-      <c r="C110" s="63"/>
-      <c r="D110" s="56"/>
-      <c r="E110" s="52"/>
-      <c r="F110" s="52"/>
-      <c r="G110" s="56"/>
-      <c r="H110" s="56"/>
-      <c r="I110" s="52"/>
-      <c r="J110" s="54"/>
-      <c r="K110" s="54"/>
-      <c r="L110" s="54"/>
-      <c r="M110" s="54"/>
-      <c r="N110" s="54"/>
-      <c r="O110" s="54"/>
-      <c r="P110" s="54"/>
-    </row>
-    <row r="111" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A111" s="54"/>
-      <c r="B111" s="52"/>
-      <c r="C111" s="52"/>
-      <c r="D111" s="52"/>
-      <c r="E111" s="52"/>
-      <c r="F111" s="52"/>
-      <c r="G111" s="52"/>
-      <c r="H111" s="52"/>
-      <c r="I111" s="52"/>
-      <c r="J111" s="54"/>
-      <c r="K111" s="54"/>
-      <c r="L111" s="54"/>
-      <c r="M111" s="54"/>
-      <c r="N111" s="54"/>
-      <c r="O111" s="54"/>
-      <c r="P111" s="54"/>
-    </row>
-    <row r="112" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A112" s="54"/>
-      <c r="B112" s="52"/>
-      <c r="C112" s="52"/>
-      <c r="D112" s="52"/>
-      <c r="E112" s="52"/>
-      <c r="F112" s="52"/>
-      <c r="G112" s="52"/>
-      <c r="H112" s="52"/>
-      <c r="I112" s="52"/>
-      <c r="J112" s="54"/>
-      <c r="K112" s="54"/>
-      <c r="L112" s="54"/>
-      <c r="M112" s="54"/>
-      <c r="N112" s="54"/>
-      <c r="O112" s="54"/>
-      <c r="P112" s="54"/>
-    </row>
-    <row r="113" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A113" s="54"/>
-      <c r="B113" s="56"/>
-      <c r="C113" s="52"/>
-      <c r="D113" s="52"/>
-      <c r="E113" s="64"/>
-      <c r="F113" s="52"/>
-      <c r="G113" s="65"/>
-      <c r="H113" s="52"/>
-      <c r="I113" s="52"/>
-      <c r="J113" s="54"/>
-      <c r="K113" s="54"/>
-      <c r="L113" s="54"/>
-      <c r="M113" s="54"/>
-      <c r="N113" s="54"/>
-      <c r="O113" s="54"/>
-      <c r="P113" s="54"/>
-    </row>
-    <row r="114" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A114" s="54"/>
-      <c r="B114" s="57"/>
-      <c r="C114" s="56"/>
-      <c r="D114" s="56"/>
-      <c r="E114" s="58"/>
-      <c r="F114" s="52"/>
-      <c r="G114" s="52"/>
-      <c r="H114" s="52"/>
-      <c r="I114" s="52"/>
-      <c r="J114" s="54"/>
-      <c r="K114" s="54"/>
-      <c r="L114" s="54"/>
-      <c r="M114" s="54"/>
-      <c r="N114" s="54"/>
-      <c r="O114" s="54"/>
-      <c r="P114" s="54"/>
-    </row>
-    <row r="115" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A115" s="54"/>
-      <c r="B115" s="56"/>
-      <c r="C115" s="66"/>
-      <c r="D115" s="66"/>
-      <c r="E115" s="56"/>
-      <c r="F115" s="52"/>
-      <c r="G115" s="52"/>
-      <c r="H115" s="52"/>
-      <c r="I115" s="52"/>
-      <c r="J115" s="54"/>
-      <c r="K115" s="54"/>
-      <c r="L115" s="54"/>
-      <c r="M115" s="54"/>
-      <c r="N115" s="54"/>
-      <c r="O115" s="54"/>
-      <c r="P115" s="54"/>
-    </row>
-    <row r="116" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A116" s="54"/>
-      <c r="B116" s="56"/>
-      <c r="C116" s="66"/>
-      <c r="D116" s="66"/>
-      <c r="E116" s="56"/>
-      <c r="F116" s="54"/>
-      <c r="G116" s="54"/>
-      <c r="H116" s="54"/>
-      <c r="I116" s="54"/>
-      <c r="J116" s="54"/>
-      <c r="K116" s="54"/>
-      <c r="L116" s="54"/>
-      <c r="M116" s="54"/>
-      <c r="N116" s="54"/>
-      <c r="O116" s="54"/>
-      <c r="P116" s="54"/>
-    </row>
-    <row r="117" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A117" s="54"/>
-      <c r="B117" s="56"/>
-      <c r="C117" s="56"/>
-      <c r="D117" s="66"/>
-      <c r="E117" s="56"/>
-      <c r="F117" s="54"/>
-      <c r="G117" s="54"/>
-      <c r="H117" s="54"/>
-      <c r="I117" s="54"/>
-      <c r="J117" s="54"/>
-      <c r="K117" s="54"/>
-      <c r="L117" s="54"/>
-      <c r="M117" s="54"/>
-      <c r="N117" s="54"/>
-      <c r="O117" s="54"/>
-      <c r="P117" s="54"/>
-    </row>
-    <row r="118" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A118" s="54"/>
-      <c r="B118" s="54"/>
-      <c r="C118" s="54"/>
-      <c r="D118" s="54"/>
-      <c r="E118" s="54"/>
-      <c r="F118" s="54"/>
-      <c r="G118" s="54"/>
-      <c r="H118" s="54"/>
-      <c r="I118" s="54"/>
-      <c r="J118" s="54"/>
-      <c r="K118" s="54"/>
-      <c r="L118" s="54"/>
-      <c r="M118" s="54"/>
-      <c r="N118" s="54"/>
-      <c r="O118" s="54"/>
-      <c r="P118" s="54"/>
-    </row>
-    <row r="119" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A119" s="54"/>
-      <c r="B119" s="52"/>
-      <c r="C119" s="54"/>
-      <c r="D119" s="54"/>
-      <c r="E119" s="54"/>
-      <c r="F119" s="54"/>
-      <c r="G119" s="54"/>
-      <c r="H119" s="54"/>
-      <c r="I119" s="54"/>
-      <c r="J119" s="54"/>
-      <c r="K119" s="54"/>
-      <c r="L119" s="54"/>
-      <c r="M119" s="54"/>
-      <c r="N119" s="54"/>
-      <c r="O119" s="54"/>
-      <c r="P119" s="54"/>
-    </row>
-    <row r="120" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A120" s="54"/>
-      <c r="B120" s="52"/>
-      <c r="C120" s="54"/>
-      <c r="D120" s="54"/>
-      <c r="E120" s="54"/>
-      <c r="F120" s="54"/>
-      <c r="G120" s="54"/>
-      <c r="H120" s="54"/>
-      <c r="I120" s="54"/>
-      <c r="J120" s="54"/>
-      <c r="K120" s="54"/>
-      <c r="L120" s="54"/>
-      <c r="M120" s="54"/>
-      <c r="N120" s="54"/>
-      <c r="O120" s="54"/>
-      <c r="P120" s="54"/>
-    </row>
-    <row r="121" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A121" s="54"/>
-      <c r="B121" s="54"/>
-      <c r="C121" s="54"/>
-      <c r="D121" s="54"/>
-      <c r="E121" s="54"/>
-      <c r="F121" s="54"/>
-      <c r="G121" s="54"/>
-      <c r="H121" s="54"/>
-      <c r="I121" s="54"/>
-      <c r="J121" s="54"/>
-      <c r="K121" s="54"/>
-      <c r="L121" s="54"/>
-      <c r="M121" s="54"/>
-      <c r="N121" s="54"/>
-      <c r="O121" s="54"/>
-      <c r="P121" s="54"/>
-    </row>
-    <row r="122" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A122" s="54"/>
-      <c r="B122" s="54"/>
-      <c r="C122" s="54"/>
-      <c r="D122" s="54"/>
-      <c r="E122" s="54"/>
-      <c r="F122" s="54"/>
-      <c r="G122" s="54"/>
-      <c r="H122" s="54"/>
-      <c r="I122" s="54"/>
-      <c r="J122" s="54"/>
-      <c r="K122" s="54"/>
-      <c r="L122" s="54"/>
-      <c r="M122" s="54"/>
-      <c r="N122" s="54"/>
-      <c r="O122" s="54"/>
-      <c r="P122" s="54"/>
-    </row>
-    <row r="123" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A123" s="54"/>
-      <c r="B123" s="54"/>
-      <c r="C123" s="54"/>
-      <c r="D123" s="54"/>
-      <c r="E123" s="54"/>
-      <c r="F123" s="54"/>
-      <c r="G123" s="54"/>
-      <c r="H123" s="54"/>
-      <c r="I123" s="54"/>
-      <c r="J123" s="54"/>
-      <c r="K123" s="54"/>
-      <c r="L123" s="54"/>
-      <c r="M123" s="54"/>
-      <c r="N123" s="54"/>
-      <c r="O123" s="54"/>
-      <c r="P123" s="54"/>
-    </row>
-    <row r="124" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A124" s="54"/>
-      <c r="B124" s="62"/>
-      <c r="C124" s="54"/>
-      <c r="D124" s="54"/>
-      <c r="E124" s="54"/>
-      <c r="F124" s="54"/>
-      <c r="G124" s="54"/>
-      <c r="H124" s="54"/>
-      <c r="I124" s="54"/>
-      <c r="J124" s="54"/>
-      <c r="K124" s="54"/>
-      <c r="L124" s="54"/>
-      <c r="M124" s="54"/>
-      <c r="N124" s="54"/>
-      <c r="O124" s="54"/>
-      <c r="P124" s="54"/>
-    </row>
-    <row r="125" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A125" s="54"/>
-      <c r="B125" s="62"/>
-      <c r="C125" s="54"/>
-      <c r="D125" s="54"/>
-      <c r="E125" s="54"/>
-      <c r="F125" s="54"/>
-      <c r="G125" s="54"/>
-      <c r="H125" s="54"/>
-      <c r="I125" s="54"/>
-      <c r="J125" s="54"/>
-      <c r="K125" s="54"/>
-      <c r="L125" s="54"/>
-      <c r="M125" s="54"/>
-      <c r="N125" s="54"/>
-      <c r="O125" s="54"/>
-      <c r="P125" s="54"/>
-    </row>
-    <row r="126" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A126" s="54"/>
-      <c r="B126" s="62"/>
-      <c r="C126" s="54"/>
-      <c r="D126" s="54"/>
-      <c r="E126" s="54"/>
-      <c r="F126" s="54"/>
-      <c r="G126" s="54"/>
-      <c r="H126" s="54"/>
-      <c r="I126" s="54"/>
-      <c r="J126" s="54"/>
-      <c r="K126" s="54"/>
-      <c r="L126" s="54"/>
-      <c r="M126" s="54"/>
-      <c r="N126" s="54"/>
-      <c r="O126" s="54"/>
-      <c r="P126" s="54"/>
-    </row>
-    <row r="127" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A127" s="54"/>
-      <c r="B127" s="54"/>
-      <c r="C127" s="54"/>
-      <c r="D127" s="54"/>
-      <c r="E127" s="54"/>
-      <c r="F127" s="54"/>
-      <c r="G127" s="54"/>
-      <c r="H127" s="54"/>
-      <c r="I127" s="54"/>
-      <c r="J127" s="54"/>
-      <c r="K127" s="54"/>
-      <c r="L127" s="54"/>
-      <c r="M127" s="54"/>
-      <c r="N127" s="54"/>
-      <c r="O127" s="54"/>
-      <c r="P127" s="54"/>
-    </row>
-    <row r="128" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A128" s="54"/>
-      <c r="B128" s="54"/>
-      <c r="C128" s="54"/>
-      <c r="D128" s="54"/>
-      <c r="E128" s="54"/>
-      <c r="F128" s="54"/>
-      <c r="G128" s="54"/>
-      <c r="H128" s="54"/>
-      <c r="I128" s="54"/>
-      <c r="J128" s="54"/>
-      <c r="K128" s="54"/>
-      <c r="L128" s="54"/>
-      <c r="M128" s="54"/>
-      <c r="N128" s="54"/>
-      <c r="O128" s="54"/>
-      <c r="P128" s="54"/>
-    </row>
-    <row r="129" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A129" s="54"/>
-      <c r="B129" s="56"/>
-      <c r="C129" s="52"/>
-      <c r="D129" s="52"/>
-      <c r="E129" s="54"/>
-      <c r="F129" s="54"/>
-      <c r="G129" s="54"/>
-      <c r="H129" s="54"/>
-      <c r="I129" s="54"/>
-      <c r="J129" s="54"/>
-      <c r="K129" s="54"/>
-      <c r="L129" s="54"/>
-      <c r="M129" s="54"/>
-      <c r="N129" s="54"/>
-      <c r="O129" s="54"/>
-      <c r="P129" s="54"/>
-    </row>
-    <row r="130" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A130" s="54"/>
-      <c r="B130" s="57"/>
-      <c r="C130" s="56"/>
-      <c r="D130" s="56"/>
-      <c r="E130" s="54"/>
-      <c r="F130" s="54"/>
-      <c r="G130" s="54"/>
-      <c r="H130" s="54"/>
-      <c r="I130" s="54"/>
-      <c r="J130" s="54"/>
-      <c r="K130" s="54"/>
-      <c r="L130" s="54"/>
-      <c r="M130" s="54"/>
-      <c r="N130" s="54"/>
-      <c r="O130" s="54"/>
-      <c r="P130" s="54"/>
-    </row>
-    <row r="131" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A131" s="54"/>
-      <c r="B131" s="56"/>
-      <c r="C131" s="56"/>
-      <c r="D131" s="56"/>
-      <c r="E131" s="54"/>
-      <c r="F131" s="54"/>
-      <c r="G131" s="54"/>
-      <c r="H131" s="54"/>
-      <c r="I131" s="54"/>
-      <c r="J131" s="54"/>
-      <c r="K131" s="54"/>
-      <c r="L131" s="54"/>
-      <c r="M131" s="54"/>
-      <c r="N131" s="54"/>
-      <c r="O131" s="54"/>
-      <c r="P131" s="54"/>
-    </row>
-    <row r="132" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A132" s="54"/>
-      <c r="B132" s="56"/>
-      <c r="C132" s="56"/>
-      <c r="D132" s="56"/>
-      <c r="E132" s="54"/>
-      <c r="F132" s="54"/>
-      <c r="G132" s="54"/>
-      <c r="H132" s="54"/>
-      <c r="I132" s="54"/>
-      <c r="J132" s="54"/>
-      <c r="K132" s="54"/>
-      <c r="L132" s="54"/>
-      <c r="M132" s="54"/>
-      <c r="N132" s="54"/>
-      <c r="O132" s="54"/>
-      <c r="P132" s="54"/>
-    </row>
-    <row r="133" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A133" s="54"/>
-      <c r="B133" s="56"/>
-      <c r="C133" s="56"/>
-      <c r="D133" s="56"/>
-      <c r="E133" s="54"/>
-      <c r="F133" s="54"/>
-      <c r="G133" s="54"/>
-      <c r="H133" s="54"/>
-      <c r="I133" s="54"/>
-      <c r="J133" s="54"/>
-      <c r="K133" s="54"/>
-      <c r="L133" s="54"/>
-      <c r="M133" s="54"/>
-      <c r="N133" s="54"/>
-      <c r="O133" s="54"/>
-      <c r="P133" s="54"/>
-    </row>
-    <row r="134" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A134" s="54"/>
-      <c r="B134" s="56"/>
-      <c r="C134" s="63"/>
-      <c r="D134" s="56"/>
-      <c r="E134" s="54"/>
-      <c r="F134" s="54"/>
-      <c r="G134" s="54"/>
-      <c r="H134" s="54"/>
-      <c r="I134" s="54"/>
-      <c r="J134" s="54"/>
-      <c r="K134" s="54"/>
-      <c r="L134" s="54"/>
-      <c r="M134" s="54"/>
-      <c r="N134" s="54"/>
-      <c r="O134" s="54"/>
-      <c r="P134" s="54"/>
-    </row>
-    <row r="135" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A135" s="54"/>
-      <c r="B135" s="54"/>
-      <c r="C135" s="54"/>
-      <c r="D135" s="54"/>
-      <c r="E135" s="54"/>
-      <c r="F135" s="54"/>
-      <c r="G135" s="54"/>
-      <c r="H135" s="54"/>
-      <c r="I135" s="54"/>
-      <c r="J135" s="54"/>
-      <c r="K135" s="54"/>
-      <c r="L135" s="54"/>
-      <c r="M135" s="54"/>
-      <c r="N135" s="54"/>
-      <c r="O135" s="54"/>
-      <c r="P135" s="54"/>
-    </row>
-    <row r="136" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A136" s="54"/>
-      <c r="B136" s="54"/>
-      <c r="C136" s="54"/>
-      <c r="D136" s="54"/>
-      <c r="E136" s="54"/>
-      <c r="F136" s="54"/>
-      <c r="G136" s="54"/>
-      <c r="H136" s="54"/>
-      <c r="I136" s="54"/>
-      <c r="J136" s="54"/>
-      <c r="K136" s="54"/>
-      <c r="L136" s="54"/>
-      <c r="M136" s="54"/>
-      <c r="N136" s="54"/>
-      <c r="O136" s="54"/>
-      <c r="P136" s="54"/>
-    </row>
-    <row r="137" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A137" s="54"/>
-      <c r="B137" s="56"/>
-      <c r="C137" s="56"/>
-      <c r="D137" s="56"/>
-      <c r="E137" s="56"/>
-      <c r="F137" s="54"/>
-      <c r="G137" s="54"/>
-      <c r="H137" s="54"/>
-      <c r="I137" s="54"/>
-      <c r="J137" s="54"/>
-      <c r="K137" s="54"/>
-      <c r="L137" s="54"/>
-      <c r="M137" s="54"/>
-      <c r="N137" s="54"/>
-      <c r="O137" s="54"/>
-      <c r="P137" s="54"/>
-    </row>
-    <row r="138" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A138" s="54"/>
-      <c r="B138" s="57"/>
-      <c r="C138" s="56"/>
-      <c r="D138" s="56"/>
-      <c r="E138" s="58"/>
-      <c r="F138" s="54"/>
-      <c r="G138" s="54"/>
-      <c r="H138" s="54"/>
-      <c r="I138" s="54"/>
-      <c r="J138" s="54"/>
-      <c r="K138" s="54"/>
-      <c r="L138" s="54"/>
-      <c r="M138" s="54"/>
-      <c r="N138" s="54"/>
-      <c r="O138" s="54"/>
-      <c r="P138" s="54"/>
-    </row>
-    <row r="139" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A139" s="54"/>
-      <c r="B139" s="56"/>
-      <c r="C139" s="56"/>
-      <c r="D139" s="56"/>
-      <c r="E139" s="56"/>
-      <c r="F139" s="54"/>
-      <c r="G139" s="54"/>
-      <c r="H139" s="54"/>
-      <c r="I139" s="54"/>
-      <c r="J139" s="54"/>
-      <c r="K139" s="54"/>
-      <c r="L139" s="54"/>
-      <c r="M139" s="54"/>
-      <c r="N139" s="54"/>
-      <c r="O139" s="54"/>
-      <c r="P139" s="54"/>
-    </row>
-    <row r="140" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A140" s="54"/>
-      <c r="B140" s="56"/>
-      <c r="C140" s="56"/>
-      <c r="D140" s="56"/>
-      <c r="E140" s="56"/>
-      <c r="F140" s="54"/>
-      <c r="G140" s="54"/>
-      <c r="H140" s="54"/>
-      <c r="I140" s="54"/>
-      <c r="J140" s="54"/>
-      <c r="K140" s="54"/>
-      <c r="L140" s="54"/>
-      <c r="M140" s="54"/>
-      <c r="N140" s="54"/>
-      <c r="O140" s="54"/>
-      <c r="P140" s="54"/>
-    </row>
-    <row r="141" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A141" s="54"/>
-      <c r="B141" s="56"/>
-      <c r="C141" s="56"/>
-      <c r="D141" s="56"/>
-      <c r="E141" s="56"/>
-      <c r="F141" s="54"/>
-      <c r="G141" s="54"/>
-      <c r="H141" s="54"/>
-      <c r="I141" s="54"/>
-      <c r="J141" s="54"/>
-      <c r="K141" s="54"/>
-      <c r="L141" s="54"/>
-      <c r="M141" s="54"/>
-      <c r="N141" s="54"/>
-      <c r="O141" s="54"/>
-      <c r="P141" s="54"/>
-    </row>
-    <row r="142" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A142" s="54"/>
-      <c r="B142" s="56"/>
-      <c r="C142" s="56"/>
-      <c r="D142" s="56"/>
-      <c r="E142" s="56"/>
-      <c r="F142" s="54"/>
-      <c r="G142" s="54"/>
-      <c r="H142" s="54"/>
-      <c r="I142" s="54"/>
-      <c r="J142" s="54"/>
-      <c r="K142" s="54"/>
-      <c r="L142" s="54"/>
-      <c r="M142" s="54"/>
-      <c r="N142" s="54"/>
-      <c r="O142" s="54"/>
-      <c r="P142" s="54"/>
-    </row>
-    <row r="143" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A143" s="54"/>
-      <c r="B143" s="56"/>
-      <c r="C143" s="56"/>
-      <c r="D143" s="56"/>
-      <c r="E143" s="56"/>
-      <c r="F143" s="54"/>
-      <c r="G143" s="54"/>
-      <c r="H143" s="54"/>
-      <c r="I143" s="54"/>
-      <c r="J143" s="54"/>
-      <c r="K143" s="54"/>
-      <c r="L143" s="54"/>
-      <c r="M143" s="54"/>
-      <c r="N143" s="54"/>
-      <c r="O143" s="54"/>
-      <c r="P143" s="54"/>
-    </row>
-    <row r="144" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A144" s="54"/>
-      <c r="B144" s="54"/>
-      <c r="C144" s="54"/>
-      <c r="D144" s="54"/>
-      <c r="E144" s="54"/>
-      <c r="F144" s="54"/>
-      <c r="G144" s="54"/>
-      <c r="H144" s="54"/>
-      <c r="I144" s="54"/>
-      <c r="J144" s="54"/>
-      <c r="K144" s="54"/>
-      <c r="L144" s="54"/>
-      <c r="M144" s="54"/>
-      <c r="N144" s="54"/>
-      <c r="O144" s="54"/>
-      <c r="P144" s="54"/>
-    </row>
-    <row r="145" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A145" s="54"/>
-      <c r="B145" s="54"/>
-      <c r="C145" s="54"/>
-      <c r="D145" s="54"/>
-      <c r="E145" s="54"/>
-      <c r="F145" s="54"/>
-      <c r="G145" s="54"/>
-      <c r="H145" s="54"/>
-      <c r="I145" s="54"/>
-      <c r="J145" s="54"/>
-      <c r="K145" s="54"/>
-      <c r="L145" s="54"/>
-      <c r="M145" s="54"/>
-      <c r="N145" s="54"/>
-      <c r="O145" s="54"/>
-      <c r="P145" s="54"/>
-    </row>
-    <row r="146" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A146" s="54"/>
-      <c r="B146" s="56"/>
-      <c r="C146" s="54"/>
-      <c r="D146" s="54"/>
-      <c r="E146" s="54"/>
-      <c r="F146" s="54"/>
-      <c r="G146" s="54"/>
-      <c r="H146" s="54"/>
-      <c r="I146" s="54"/>
-      <c r="J146" s="54"/>
-      <c r="K146" s="54"/>
-      <c r="L146" s="54"/>
-      <c r="M146" s="54"/>
-      <c r="N146" s="54"/>
-      <c r="O146" s="54"/>
-      <c r="P146" s="54"/>
-    </row>
-    <row r="147" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B147" s="50" t="s">
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C49" s="25"/>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C50" s="25"/>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="I55" s="29"/>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="I56" s="29"/>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="I57" s="29"/>
+    </row>
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A58" s="39"/>
+      <c r="B58" s="29"/>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A59" s="39"/>
+      <c r="B59" s="29"/>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A60" s="39"/>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A61" s="39"/>
+      <c r="B61" s="29"/>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A62" s="39"/>
+      <c r="B62" s="29"/>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" s="39"/>
+      <c r="B63" s="29"/>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B64" s="31"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="31"/>
+      <c r="I64" s="31"/>
+      <c r="J64" s="31"/>
+      <c r="K64" s="31"/>
+      <c r="M64" s="31"/>
+    </row>
+    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B65" s="50"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="I65" s="50"/>
+      <c r="J65" s="31"/>
+      <c r="K65" s="31"/>
+      <c r="M65" s="51"/>
+      <c r="N65" s="51"/>
+    </row>
+    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B66" s="31"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="I66" s="31"/>
+      <c r="J66" s="31"/>
+      <c r="K66" s="31"/>
+      <c r="M66" s="31"/>
+      <c r="N66" s="31"/>
+    </row>
+    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B67" s="31"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="I67" s="31"/>
+      <c r="J67" s="31"/>
+      <c r="K67" s="31"/>
+      <c r="M67" s="31"/>
+      <c r="N67" s="31"/>
+    </row>
+    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B68" s="31"/>
+      <c r="C68" s="31"/>
+      <c r="D68" s="31"/>
+      <c r="I68" s="31"/>
+      <c r="J68" s="31"/>
+      <c r="K68" s="31"/>
+      <c r="M68" s="31"/>
+      <c r="N68" s="31"/>
+    </row>
+    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="I69" s="31"/>
+      <c r="J69" s="31"/>
+      <c r="K69" s="31"/>
+      <c r="M69" s="31"/>
+      <c r="N69" s="31"/>
+    </row>
+    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="M70" s="31"/>
+      <c r="N70" s="31"/>
+    </row>
+    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B72" s="31"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="F72" s="31"/>
+      <c r="I72" s="31"/>
+      <c r="J72" s="31"/>
+      <c r="K72" s="31"/>
+    </row>
+    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B73" s="50"/>
+      <c r="C73" s="31"/>
+      <c r="D73" s="31"/>
+      <c r="E73" s="31"/>
+      <c r="F73" s="51"/>
+      <c r="I73" s="50"/>
+      <c r="J73" s="31"/>
+      <c r="K73" s="31"/>
+    </row>
+    <row r="74" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B74" s="31"/>
+      <c r="C74" s="31"/>
+      <c r="D74" s="31"/>
+      <c r="E74" s="31"/>
+      <c r="F74" s="31"/>
+      <c r="I74" s="31"/>
+      <c r="J74" s="31"/>
+      <c r="K74" s="31"/>
+    </row>
+    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B75" s="31"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="31"/>
+      <c r="E75" s="31"/>
+      <c r="F75" s="31"/>
+      <c r="I75" s="31"/>
+      <c r="J75" s="31"/>
+      <c r="K75" s="31"/>
+    </row>
+    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B76" s="31"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="31"/>
+      <c r="F76" s="31"/>
+      <c r="I76" s="31"/>
+      <c r="J76" s="31"/>
+      <c r="K76" s="31"/>
+    </row>
+    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B77" s="31"/>
+      <c r="C77" s="31"/>
+      <c r="D77" s="31"/>
+      <c r="E77" s="31"/>
+      <c r="F77" s="31"/>
+      <c r="I77" s="31"/>
+      <c r="J77" s="31"/>
+      <c r="K77" s="31"/>
+    </row>
+    <row r="78" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B78" s="31"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="31"/>
+      <c r="F78" s="31"/>
+    </row>
+    <row r="81" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B81" s="31"/>
+      <c r="C81" s="54"/>
+      <c r="D81" s="54"/>
+    </row>
+    <row r="82" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B82" s="50"/>
+      <c r="C82" s="31"/>
+      <c r="D82" s="31"/>
+      <c r="E82" s="31"/>
+      <c r="F82" s="52"/>
+      <c r="I82" s="31"/>
+      <c r="J82" s="31"/>
+      <c r="K82" s="31"/>
+    </row>
+    <row r="83" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B83" s="31"/>
+      <c r="C83" s="31"/>
+      <c r="D83" s="31"/>
+      <c r="E83" s="31"/>
+      <c r="F83" s="31"/>
+      <c r="I83" s="50"/>
+      <c r="J83" s="31"/>
+      <c r="K83" s="51"/>
+    </row>
+    <row r="84" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B84" s="31"/>
+      <c r="C84" s="31"/>
+      <c r="D84" s="31"/>
+      <c r="E84" s="31"/>
+      <c r="F84" s="31"/>
+      <c r="I84" s="31"/>
+      <c r="J84" s="31"/>
+      <c r="K84" s="31"/>
+    </row>
+    <row r="85" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B85" s="31"/>
+      <c r="C85" s="31"/>
+      <c r="D85" s="31"/>
+      <c r="E85" s="31"/>
+      <c r="F85" s="31"/>
+      <c r="I85" s="31"/>
+      <c r="J85" s="31"/>
+      <c r="K85" s="31"/>
+    </row>
+    <row r="86" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B86" s="31"/>
+      <c r="C86" s="31"/>
+      <c r="D86" s="31"/>
+      <c r="E86" s="31"/>
+      <c r="F86" s="31"/>
+      <c r="I86" s="31"/>
+      <c r="J86" s="31"/>
+      <c r="K86" s="31"/>
+    </row>
+    <row r="87" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B87" s="31"/>
+      <c r="C87" s="31"/>
+      <c r="D87" s="31"/>
+      <c r="E87" s="31"/>
+      <c r="F87" s="31"/>
+      <c r="I87" s="31"/>
+      <c r="J87" s="31"/>
+      <c r="K87" s="31"/>
+    </row>
+    <row r="88" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B88" s="31"/>
+      <c r="C88" s="31"/>
+      <c r="D88" s="31"/>
+      <c r="E88" s="31"/>
+      <c r="F88" s="31"/>
+      <c r="I88" s="31"/>
+      <c r="J88" s="31"/>
+      <c r="K88" s="31"/>
+    </row>
+    <row r="89" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I89" s="31"/>
+      <c r="J89" s="31"/>
+      <c r="K89" s="31"/>
+    </row>
+    <row r="90" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I90" s="31"/>
+      <c r="J90" s="31"/>
+      <c r="K90" s="31"/>
+    </row>
+    <row r="91" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B91" s="31"/>
+      <c r="C91" s="31"/>
+      <c r="I91" s="31"/>
+      <c r="J91" s="31"/>
+      <c r="K91" s="31"/>
+    </row>
+    <row r="92" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B92" s="50"/>
+      <c r="C92" s="51"/>
+      <c r="D92" s="52"/>
+    </row>
+    <row r="93" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B93" s="31"/>
+      <c r="C93" s="31"/>
+      <c r="D93" s="31"/>
+    </row>
+    <row r="94" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B94" s="31"/>
+      <c r="C94" s="31"/>
+      <c r="D94" s="31"/>
+    </row>
+    <row r="95" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B95" s="31"/>
+      <c r="C95" s="31"/>
+      <c r="D95" s="31"/>
+    </row>
+    <row r="96" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B96" s="31"/>
+      <c r="C96" s="31"/>
+      <c r="D96" s="31"/>
+    </row>
+    <row r="97" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B97" s="31"/>
+      <c r="C97" s="31"/>
+      <c r="D97" s="31"/>
+    </row>
+    <row r="98" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B98" s="31"/>
+      <c r="C98" s="31"/>
+      <c r="D98" s="31"/>
+    </row>
+    <row r="102" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B102" s="29"/>
+    </row>
+    <row r="103" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B103" s="29"/>
+    </row>
+    <row r="105" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B105" s="29"/>
+    </row>
+    <row r="106" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="G106" s="31"/>
+      <c r="H106" s="31"/>
+    </row>
+    <row r="107" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B107" s="31"/>
+      <c r="G107" s="31"/>
+      <c r="H107" s="31"/>
+      <c r="I107" s="31"/>
+    </row>
+    <row r="108" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B108" s="50"/>
+      <c r="C108" s="31"/>
+      <c r="D108" s="31"/>
+      <c r="G108" s="51"/>
+      <c r="H108" s="51"/>
+      <c r="I108" s="51"/>
+    </row>
+    <row r="109" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B109" s="31"/>
+      <c r="C109" s="31"/>
+      <c r="D109" s="31"/>
+      <c r="G109" s="31"/>
+      <c r="H109" s="31"/>
+      <c r="I109" s="31"/>
+    </row>
+    <row r="110" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B110" s="31"/>
+      <c r="C110" s="31"/>
+      <c r="D110" s="31"/>
+      <c r="G110" s="31"/>
+      <c r="H110" s="31"/>
+      <c r="I110" s="31"/>
+    </row>
+    <row r="111" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B111" s="31"/>
+      <c r="C111" s="31"/>
+      <c r="D111" s="31"/>
+      <c r="G111" s="31"/>
+      <c r="H111" s="31"/>
+      <c r="I111" s="31"/>
+    </row>
+    <row r="112" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B112" s="31"/>
+      <c r="C112" s="25"/>
+      <c r="D112" s="31"/>
+      <c r="G112" s="31"/>
+      <c r="H112" s="31"/>
+      <c r="I112" s="31"/>
+    </row>
+    <row r="115" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B115" s="31"/>
+      <c r="E115" s="44"/>
+      <c r="G115" s="28"/>
+      <c r="H115" s="28"/>
+    </row>
+    <row r="116" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B116" s="50"/>
+      <c r="C116" s="31"/>
+      <c r="D116" s="31"/>
+      <c r="E116" s="51"/>
+    </row>
+    <row r="117" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B117" s="31"/>
+      <c r="C117" s="53"/>
+      <c r="D117" s="53"/>
+      <c r="E117" s="31"/>
+    </row>
+    <row r="118" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B118" s="31"/>
+      <c r="C118" s="53"/>
+      <c r="D118" s="53"/>
+      <c r="E118" s="31"/>
+    </row>
+    <row r="119" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B119" s="31"/>
+      <c r="C119" s="31"/>
+      <c r="D119" s="53"/>
+      <c r="E119" s="31"/>
+    </row>
+    <row r="126" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B126" s="29"/>
+    </row>
+    <row r="127" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B127" s="29"/>
+    </row>
+    <row r="128" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B128" s="29"/>
+    </row>
+    <row r="131" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B131" s="31"/>
+    </row>
+    <row r="132" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B132" s="50"/>
+      <c r="C132" s="31"/>
+      <c r="D132" s="31"/>
+    </row>
+    <row r="133" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B133" s="31"/>
+      <c r="C133" s="31"/>
+      <c r="D133" s="31"/>
+    </row>
+    <row r="134" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B134" s="31"/>
+      <c r="C134" s="31"/>
+      <c r="D134" s="31"/>
+    </row>
+    <row r="135" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B135" s="31"/>
+      <c r="C135" s="31"/>
+      <c r="D135" s="31"/>
+    </row>
+    <row r="136" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B136" s="31"/>
+      <c r="C136" s="25"/>
+      <c r="D136" s="31"/>
+    </row>
+    <row r="139" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B139" s="31"/>
+      <c r="C139" s="31"/>
+      <c r="D139" s="31"/>
+      <c r="E139" s="31"/>
+    </row>
+    <row r="140" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B140" s="50"/>
+      <c r="C140" s="31"/>
+      <c r="D140" s="31"/>
+      <c r="E140" s="51"/>
+    </row>
+    <row r="141" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B141" s="31"/>
+      <c r="C141" s="31"/>
+      <c r="D141" s="31"/>
+      <c r="E141" s="31"/>
+    </row>
+    <row r="142" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B142" s="31"/>
+      <c r="C142" s="31"/>
+      <c r="D142" s="31"/>
+      <c r="E142" s="31"/>
+    </row>
+    <row r="143" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B143" s="31"/>
+      <c r="C143" s="31"/>
+      <c r="D143" s="31"/>
+      <c r="E143" s="31"/>
+    </row>
+    <row r="144" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B144" s="31"/>
+      <c r="C144" s="31"/>
+      <c r="D144" s="31"/>
+      <c r="E144" s="31"/>
+    </row>
+    <row r="145" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B145" s="31"/>
+      <c r="C145" s="31"/>
+      <c r="D145" s="31"/>
+      <c r="E145" s="31"/>
+    </row>
+    <row r="148" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B148" s="31"/>
+    </row>
+    <row r="149" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B149" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="C147" s="50" t="s">
+      <c r="C149" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="D147" s="51" t="s">
+      <c r="D149" s="49" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="148" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B148" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="C148" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="D148" s="33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="149" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B149" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="C149" s="33" t="s">
-        <v>137</v>
-      </c>
-      <c r="D149" s="33">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="150" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B150" s="33" t="s">
         <v>171</v>
       </c>
       <c r="C150" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D150" s="33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="151" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B151" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="C151" s="33" t="s">
+        <v>137</v>
+      </c>
+      <c r="D151" s="33">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="152" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B152" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="C152" s="33" t="s">
         <v>140</v>
-      </c>
-      <c r="D150" s="33">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="151" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B151" s="33" t="s">
-        <v>172</v>
-      </c>
-      <c r="C151" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="D151" s="33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="B152" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="C152" s="33" t="s">
-        <v>134</v>
       </c>
       <c r="D152" s="33">
         <v>2</v>
       </c>
     </row>
+    <row r="153" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B153" s="33" t="s">
+        <v>172</v>
+      </c>
+      <c r="C153" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D153" s="33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B154" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="C154" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="D154" s="33">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="C79:D79"/>
+    <mergeCell ref="C81:D81"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>